<commit_message>
Update dashboard and reports with 9-12-PD booking data
- build_dashboard.py: can now read the source .xls directly and
  compute balances itself (reuses build_booking_balance_report's
  logic), no longer requires opening the .xlsx in Excel first
- Regenerate Booking Balance Summary.xlsx, per-pickup files, and
  the dashboard from "9-12-PD - Copy.xls" (90 BK No outstanding,
  219 containers)
- README: reflect the new direct-from-.xls workflow and public
  repo status

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - B.C. DEPOT CO.,LTD. ( Bang-Na KM.18).xlsx
+++ b/output/bkg pending - B.C. DEPOT CO.,LTD. ( Bang-Na KM.18).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Pending" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$2:$AI$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$2:$AI$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -469,7 +469,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI23"/>
+  <dimension ref="A1:AI22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -730,22 +730,22 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260800103</t>
+          <t>HASLS22260702080</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>SWIC</t>
+          <t>DJCF</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>0151N</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>202609221500</t>
+          <t>202609190700</t>
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
@@ -761,41 +761,41 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>20260815</t>
+          <t>20260912</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>QUANTERM LOGISTICS (THAILAND) CO., LTD.</t>
+          <t>EAST-LINK CORPORATION CO., LTD.</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>THAI GYPSUM PRODUCTS PCL.</t>
+          <t>ABD KHAN CO., LTD</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>GYPSUM PLASTER - 25202090</t>
+          <t>MACKEREL IN TOMATO SAUCE</t>
         </is>
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>RQS CONTAINER GRADE-A FOR FOOD COMMODITY.</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
         <is>
-          <t>Pickup : 2026-08-15, Return : 2026-08-17 (1ST RTN DD: 18/09/26 WO/RENT)</t>
+          <t>Pickup : 2026-09-12, Return : 2026-09-14</t>
         </is>
       </c>
       <c r="O3" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P3" s="4" t="n">
         <v>0</v>
@@ -871,22 +871,22 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801132</t>
+          <t>HASLS22260800103</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>SWMM</t>
+          <t>SWIC</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>202609230700</t>
+          <t>202609211300</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr"/>
@@ -897,52 +897,52 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>JPMYJ</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>20260908</t>
+          <t>20260815</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>C.P. INTERTRADE CO., LTD.</t>
+          <t>QUANTERM LOGISTICS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>PERFECT COMPANION GROUP CO., LTD.</t>
+          <t>THAI GYPSUM PRODUCTS PCL.</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>PET FOOD</t>
+          <t>GYPSUM PLASTER - 25202090</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>REQ CLEAN AND GOOD CNTR STRONG FLOOR</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pickup : 2026-09-08, Return : 2026-09-09 </t>
+          <t>Pickup : 2026-08-15, Return : 2026-08-17 (1ST RTN DD: 18/09/26 WO/RENT)</t>
         </is>
       </c>
       <c r="O4" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q4" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R4" s="4" t="n">
         <v>0</v>
@@ -1012,37 +1012,33 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801433</t>
+          <t>HASLS22260800603</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>NSSJ</t>
+          <t>KMTP</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>2607S</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>202609222100</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>THLKR</t>
-        </is>
-      </c>
+          <t>202609200900</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr"/>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>THLCH</t>
+          <t>THBKK</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>IDJKT</t>
+          <t>CNXMN</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
@@ -1052,33 +1048,32 @@
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>20260904</t>
+          <t>20260910</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>SCGJWD LOGISTICS PUBLIC COMPANY LIMITED</t>
+          <t>FIRST-CLASS LOGISTICS CO., LTD.</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>NORITAKE SCG PLASTER CO., LTD.</t>
+          <t>LEE TA RUBBER TREE (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>MOULDING PLASTER</t>
+          <t xml:space="preserve">RECLIAMED RUBBER </t>
         </is>
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>good and clean cont., no oil, no rusty</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>CY-RTN : 04-07/09/2026 Paperless Code 2835
-Closing Time LKB 2026-09-27 @ 23.59 // REF : ** PT Indoporcelain **</t>
+          <t xml:space="preserve">Pickup : 2026-09-10, Return : 2026-09-12 </t>
         </is>
       </c>
       <c r="O5" s="4" t="n">
@@ -1158,22 +1153,22 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801612</t>
+          <t>HASLS22260801132</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>CMA</t>
+          <t>SWMM</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>2614N</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>202609240800</t>
+          <t>202609230700</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr"/>
@@ -1184,12 +1179,12 @@
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>JPMYJ</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
@@ -1199,37 +1194,37 @@
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>ONE WORLD LOGISTICS AND FREIGHT CO., LTD.</t>
+          <t>C.P. INTERTRADE CO., LTD.</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>DUNI (THAILAND) CO., LTD.</t>
+          <t>PERFECT COMPANION GROUP CO., LTD.</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAPER NAPKIN </t>
+          <t>PET FOOD</t>
         </is>
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>REQ. GOOD GRADE CONTAINER</t>
+          <t>REQ CLEAN AND GOOD CNTR STRONG FLOOR</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>Pickup : 2026-09-08, Return : 2026-09-09</t>
+          <t xml:space="preserve">Pickup : 2026-09-08, Return : 2026-09-09 </t>
         </is>
       </c>
       <c r="O6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="R6" s="4" t="n">
         <v>0</v>
@@ -1299,12 +1294,12 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801620</t>
+          <t>HASLS22260801170</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>SWSR</t>
+          <t>SWIC</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
@@ -1314,7 +1309,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>202609171100</t>
+          <t>202609211300</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr"/>
@@ -1325,52 +1320,52 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>KRKAN</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx4 </t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>20260907</t>
+          <t>20260912</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>SONIC INTERFREIGHT PUBLIC COMPANY LIMITED</t>
+          <t>HARPERS SEA FREIGHT CO., LTD.</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>THAI OTSUKA PHARMACEUTICAL CO., LTD.</t>
+          <t>THAI ASAHI CO., LTD.</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>MEDICAL</t>
+          <t xml:space="preserve">POTATO STARCH </t>
         </is>
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>GOOD &amp; CLEAN CONT. NO SMELL</t>
+          <t>Grade A and food grade container</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pickup : 2026-09-07, Return : 2026-09-08  </t>
+          <t>Pickup : 2026-09-12, Return : 2026-09-18</t>
         </is>
       </c>
       <c r="O7" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P7" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q7" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R7" s="4" t="n">
         <v>0</v>
@@ -1440,12 +1435,12 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801621</t>
+          <t>HASLS22260801252</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>SWSR</t>
+          <t>KJT</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1455,7 +1450,7 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>202609171100</t>
+          <t>202609210600</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr"/>
@@ -1471,41 +1466,42 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">20'x4 </t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>20260907</t>
+          <t>20260910</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>SONIC INTERFREIGHT PUBLIC COMPANY LIMITED</t>
+          <t>DSV AIR &amp; SEA LTD.</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>THAI OTSUKA PHARMACEUTICAL CO., LTD.</t>
+          <t>CHEVRON (THAILAND) LIMITED</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>MEDICAL</t>
+          <t>LUBE OIL</t>
         </is>
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>GOOD &amp; CLEAN CONT. NO SMELL</t>
+          <t>Req. Container condition  GRADE B+ CNTR / CLEAN CNTR WITH GOOD CONDITION / NO SMELL/NODAMAGES / STRONG &amp; SMOOTH FLOOR / NO NAILS / LOAD UNDERDECK</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pickup : 2026-09-07, Return : 2026-09-08 </t>
+          <t xml:space="preserve">Pickup : 2026-09-10, Return : 2026-09-11  (1ST RTN 11/09 W/O RENT) 
+ </t>
         </is>
       </c>
       <c r="O8" s="4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="P8" s="4" t="n">
         <v>0</v>
@@ -1581,33 +1577,37 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801622</t>
+          <t>HASLS22260801433</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>SWSR</t>
+          <t>NSSJ</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2607S</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>202609171100</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="inlineStr"/>
+          <t>202609232100</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>THLKR</t>
+        </is>
+      </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
@@ -1617,32 +1617,33 @@
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>20260909</t>
+          <t>20260904</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>SONIC INTERFREIGHT PUBLIC COMPANY LIMITED</t>
+          <t>SCGJWD LOGISTICS PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>THAI OTSUKA PHARMACEUTICAL CO., LTD.</t>
+          <t>NORITAKE SCG PLASTER CO., LTD.</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>MEDICAL</t>
+          <t>MOULDING PLASTER</t>
         </is>
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>GOOD &amp; CLEAN CONT. NO SMELL</t>
+          <t>good and clean cont., no oil, no rusty</t>
         </is>
       </c>
       <c r="N9" s="4" t="inlineStr">
         <is>
-          <t>Pickup : 2026-09-09, Return : 2026-09-10</t>
+          <t>CY-RTN : 04-07/09/2026 Paperless Code 2835
+Closing Time LKB 2026-09-27 @ 23.59 // REF : ** PT Indoporcelain **</t>
         </is>
       </c>
       <c r="O9" s="4" t="n">
@@ -1722,12 +1723,12 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801623</t>
+          <t>HASLS22260801454</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>SWSR</t>
+          <t>KJT</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1737,7 +1738,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>202609171100</t>
+          <t>202609210600</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr"/>
@@ -1748,52 +1749,52 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>JPTMK</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>20260908</t>
+          <t>20260910</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>SONIC INTERFREIGHT PUBLIC COMPANY LIMITED</t>
+          <t>NIPPON EXPRESS LOGISTICS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t>THAI OTSUKA PHARMACEUTICAL CO., LTD.</t>
+          <t>NIPRO (THAILAND) CORPORATION LIMITED</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>MEDICAL</t>
+          <t>MEDICAL PRODUCT</t>
         </is>
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>GOOD &amp; CLEAN CONT. NO SMELL</t>
+          <t>GOOD CONTAINER A</t>
         </is>
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>Pickup : 2026-09-08, Return : 2026-09-09</t>
+          <t>Pickup : 2026-09-10, Return : 2026-09-11 (1ST RTN DD: 12/09/26 WO/RENT)</t>
         </is>
       </c>
       <c r="O10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="R10" s="4" t="n">
         <v>0</v>
@@ -1863,33 +1864,37 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801624</t>
+          <t>HASLS22260801587</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>SWSR</t>
+          <t>NSSJ</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2607S</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>202609171100</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr"/>
+          <t>202609232100</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>THLKR</t>
+        </is>
+      </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1899,32 +1904,33 @@
       </c>
       <c r="I11" s="4" t="inlineStr">
         <is>
-          <t>20260908</t>
+          <t>20260912</t>
         </is>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
-          <t>SONIC INTERFREIGHT PUBLIC COMPANY LIMITED</t>
+          <t>KTC GLOBAL LOGISTICS CO., LTD.</t>
         </is>
       </c>
       <c r="K11" s="4" t="inlineStr">
         <is>
-          <t>THAI OTSUKA PHARMACEUTICAL CO., LTD.</t>
+          <t>MEDIFOODS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>MEDICAL</t>
+          <t>ORGANIC JASMINE RICE FLOUR 120MESH</t>
         </is>
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>GOOD &amp; CLEAN CONT. NO SMELL</t>
+          <t>GOOD &amp; CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="N11" s="4" t="inlineStr">
         <is>
-          <t>Pickup : 2026-09-08, Return : 2026-09-09</t>
+          <t>Pickup : 2026-09-12, Return : 2026-09-14 Paperless Code 2835
+Closing Time LKB 2026-09-15 @ 23.59</t>
         </is>
       </c>
       <c r="O11" s="4" t="n">
@@ -2004,22 +2010,22 @@
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801625</t>
+          <t>HASLS22260801612</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>SWSR</t>
+          <t>CMA</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2614N</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>202609171100</t>
+          <t>202609241500</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr"/>
@@ -2045,22 +2051,22 @@
       </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>SONIC INTERFREIGHT PUBLIC COMPANY LIMITED</t>
+          <t>ONE WORLD LOGISTICS AND FREIGHT CO., LTD.</t>
         </is>
       </c>
       <c r="K12" s="4" t="inlineStr">
         <is>
-          <t>THAI OTSUKA PHARMACEUTICAL CO., LTD.</t>
+          <t>DUNI (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>MEDICAL</t>
+          <t xml:space="preserve">PAPER NAPKIN </t>
         </is>
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>GOOD &amp; CLEAN CONT. NO SMELL</t>
+          <t>REQ. GOOD GRADE CONTAINER</t>
         </is>
       </c>
       <c r="N12" s="4" t="inlineStr">
@@ -2145,7 +2151,7 @@
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801739</t>
+          <t>HASLS22260801625</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -2160,7 +2166,7 @@
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>202609171100</t>
+          <t>202609181000</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr"/>
@@ -2181,32 +2187,32 @@
       </c>
       <c r="I13" s="4" t="inlineStr">
         <is>
-          <t>20260907</t>
+          <t>20260908</t>
         </is>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>KUEHNE + NAGEL LIMITED</t>
+          <t>SONIC INTERFREIGHT PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K13" s="4" t="inlineStr">
         <is>
-          <t>CITY FARM INTERFOOD CO., LTD.</t>
+          <t>THAI OTSUKA PHARMACEUTICAL CO., LTD.</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>CANNED COCONUT WATER</t>
+          <t>MEDICAL</t>
         </is>
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>Req Food grade container</t>
+          <t>GOOD &amp; CLEAN CONT. NO SMELL</t>
         </is>
       </c>
       <c r="N13" s="4" t="inlineStr">
         <is>
-          <t>Pickup : 2026-09-07, Return : 2026-09-09</t>
+          <t>Pickup : 2026-09-08, Return : 2026-09-09</t>
         </is>
       </c>
       <c r="O13" s="4" t="n">
@@ -2286,22 +2292,22 @@
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801752</t>
+          <t>HASLS22260801726</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>SWSR</t>
+          <t>PGPO</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>202609171100</t>
+          <t>202609220830</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr"/>
@@ -2312,52 +2318,52 @@
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>KRKAN</t>
         </is>
       </c>
       <c r="H14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
         <is>
-          <t>20260905</t>
+          <t>20260912</t>
         </is>
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>CARDINAL MARITIME (THAILAND) CO., LTD.</t>
+          <t>HARPERS SEA FREIGHT CO., LTD.</t>
         </is>
       </c>
       <c r="K14" s="4" t="inlineStr">
         <is>
-          <t>HERITAGE SNACKS &amp; FOOD CO., LTD.</t>
+          <t>THAI ASAHI CO., LTD.</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>NUTS</t>
+          <t xml:space="preserve">POTATO STARCH </t>
         </is>
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>Request food grade container</t>
+          <t>Grade A and food grade container</t>
         </is>
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>Pickup : 2026-09-05, Return : 2026-09-07 *1ST RETURN CNTR DD.13/09/2026 WITHOUT RENT*</t>
+          <t xml:space="preserve">Pickup : 2026-09-12, Return : 2026-09-17 </t>
         </is>
       </c>
       <c r="O14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="P14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="R14" s="4" t="n">
         <v>0</v>
@@ -2427,22 +2433,22 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801927</t>
+          <t>HASLS22260801869</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>DJCF</t>
+          <t>KJT</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>0151N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>202609190200</t>
+          <t>202609210600</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr"/>
@@ -2453,52 +2459,52 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>KRINC</t>
+          <t>CNSHK</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>20260909</t>
+          <t>20260910</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>ORIENTAL LOGISTICS GROUP (THAILAND) CO., LTD.</t>
+          <t>DIMERCO EXPRESS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>KINGBOARD LAMINATE MANUFACTURING (THAILAND) CO., LTD.</t>
+          <t>THAIMAN INDUSTRIES CO., LTD.</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>LAMINATE</t>
+          <t>MULTIPLE YARN OF POLYESTER</t>
         </is>
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>request a grade container</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>Pickup : 2026-09-09, Return : 2026-09-10</t>
+          <t>Pickup : 2026-09-10, Return : 2026-09-11</t>
         </is>
       </c>
       <c r="O15" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P15" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q15" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R15" s="4" t="n">
         <v>0</v>
@@ -2568,22 +2574,22 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801939</t>
+          <t>HASLS22260801927</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>SWBT</t>
+          <t>DJCF</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>2615N</t>
+          <t>0151N</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>202609201230</t>
+          <t>202609190700</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr"/>
@@ -2594,52 +2600,52 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>KRINC</t>
         </is>
       </c>
       <c r="H16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>20260905</t>
+          <t>20260909</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
         <is>
-          <t>QUANTERM LOGISTICS (THAILAND) CO., LTD.</t>
+          <t>ORIENTAL LOGISTICS GROUP (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K16" s="4" t="inlineStr">
         <is>
-          <t>VISTA DISTRIBUTION CO.,LTD.</t>
+          <t>KINGBOARD LAMINATE MANUFACTURING (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>SNACK</t>
+          <t>LAMINATE</t>
         </is>
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>request a grade container</t>
         </is>
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>Pickup : 2026-09-05, Return : 2026-09-07 (1ST RTN DD: 13/09/26 WO/RENT)</t>
+          <t>Pickup : 2026-09-09, Return : 2026-09-10</t>
         </is>
       </c>
       <c r="O16" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P16" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q16" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R16" s="4" t="n">
         <v>0</v>
@@ -2709,22 +2715,22 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260802132</t>
+          <t>HASLS22260801939</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>SWSR</t>
+          <t>SWBT</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2615N</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>202609171100</t>
+          <t>202609211700</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr"/>
@@ -2735,32 +2741,32 @@
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>CNXMN</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>20260909</t>
+          <t>20260905</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>MARCH LOGISTICS CO., LTD.</t>
+          <t>QUANTERM LOGISTICS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>STARPRO PTR STARCH (THAILAND) CO., LTD.</t>
+          <t>VISTA DISTRIBUTION CO.,LTD.</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>STARCH</t>
+          <t>SNACK</t>
         </is>
       </c>
       <c r="M17" s="4" t="inlineStr">
@@ -2770,17 +2776,17 @@
       </c>
       <c r="N17" s="4" t="inlineStr">
         <is>
-          <t>Pickup : 2026-09-09, Return : 2026-09-14</t>
+          <t>Pickup : 2026-09-05, Return : 2026-09-07 (1ST RTN DD: 13/09/26 WO/RENT)</t>
         </is>
       </c>
       <c r="O17" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q17" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R17" s="4" t="n">
         <v>0</v>
@@ -2801,7 +2807,7 @@
         <v>0</v>
       </c>
       <c r="X17" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y17" s="4" t="n">
         <v>0</v>
@@ -2850,22 +2856,22 @@
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260802380</t>
+          <t>HASLS22260802240</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>KUS</t>
+          <t>KMTP</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>2615N</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>202609220300</t>
+          <t>202609200900</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr"/>
@@ -2876,32 +2882,32 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>KRINC</t>
+          <t>CNXMN</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x6 </t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>20260903</t>
+          <t>20260912</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>JGL WORLDWIDE (THAILAND) CO., LTD.</t>
+          <t>MARCH LOGISTICS CO., LTD.</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>ASIAN FOODS CO.,LTD.</t>
+          <t>STARPRO STARCH (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">KRISPY ROLL </t>
+          <t>STARCH</t>
         </is>
       </c>
       <c r="M18" s="4" t="inlineStr">
@@ -2911,17 +2917,17 @@
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>Pickup : 2026-09-03, Return : 2026-09-04 (1ST RTN DD: 17/09/26 WO/RENT)</t>
+          <t xml:space="preserve">Pickup : 2026-09-12, Return : 2026-09-16 </t>
         </is>
       </c>
       <c r="O18" s="4" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="P18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q18" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R18" s="4" t="n">
         <v>0</v>
@@ -2991,22 +2997,22 @@
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260802441</t>
+          <t>HASLS22260802380</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>SWSR</t>
+          <t>KUS</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2615N</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>202609171100</t>
+          <t>202609222100</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr"/>
@@ -3017,52 +3023,52 @@
       </c>
       <c r="G19" s="4" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>KRINC</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I19" s="4" t="inlineStr">
         <is>
-          <t>20260908</t>
+          <t>20260903</t>
         </is>
       </c>
       <c r="J19" s="4" t="inlineStr">
         <is>
-          <t>QONATUS SERVICE CO., LTD.</t>
+          <t>JGL WORLDWIDE (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K19" s="4" t="inlineStr">
         <is>
-          <t>AB FOOD &amp; BEVERAGES (THAILAND) LTD.</t>
+          <t>ASIAN FOODS CO.,LTD.</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>BEVERAGE</t>
+          <t xml:space="preserve">KRISPY ROLL </t>
         </is>
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>GOOD &amp; CLEAN CNTR</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>Pickup : 2026-09-08, Return : 2026-09-09 *1ST RETURN CNTR DD.13/09/2026*</t>
+          <t>Pickup : 2026-09-03, Return : 2026-09-04 (1ST RTN DD: 17/09/26 WO/RENT)</t>
         </is>
       </c>
       <c r="O19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="P19" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="R19" s="4" t="n">
         <v>0</v>
@@ -3132,22 +3138,22 @@
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260900475</t>
+          <t>HASLS22260900134</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>DJCF</t>
+          <t>KJT</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>0151N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>202609190200</t>
+          <t>202609210600</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr"/>
@@ -3158,17 +3164,17 @@
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>HKHKG</t>
         </is>
       </c>
       <c r="H20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx5 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>20260908</t>
+          <t>20260912</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -3178,32 +3184,32 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>ASIAN-PACIFIC CAN CO., LTD.</t>
+          <t>THAI PLASPAC PUBLIC CO.,LTD.</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">EMPTY CAN </t>
+          <t>PLASTIC CAP</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>**REQUEST CLEAN AND GOOD CONTAINER</t>
         </is>
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>Pickup : 2026-09-08, Return : 2026-09-14 / FIRST DATE CAN RETURN CNTR DD.14/09 WITHOUT RENT</t>
+          <t>Pickup : 2026-09-12, Return : 2026-09-14</t>
         </is>
       </c>
       <c r="O20" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P20" s="4" t="n">
         <v>0</v>
       </c>
       <c r="Q20" s="4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="R20" s="4" t="n">
         <v>0</v>
@@ -3273,22 +3279,22 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260900486</t>
+          <t>HASLS22260900475</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>KJT</t>
+          <t>DJCF</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>0151N</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>202609202200</t>
+          <t>202609190700</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr"/>
@@ -3299,12 +3305,12 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>TWKEL</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx2 </t>
+          <t xml:space="preserve">40Hx5 </t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
@@ -3314,17 +3320,17 @@
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>MORRISON EXPRESS CORP (THAILAND)LTD.</t>
+          <t>ACCORD PILOT LOGISTICS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>DELTA ELECTRONICS (THAILAND) PUBLIC COMPANY LIMITED</t>
+          <t>ASIAN-PACIFIC CAN CO., LTD.</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>ELECTRONICS COMPONENT</t>
+          <t xml:space="preserve">EMPTY CAN </t>
         </is>
       </c>
       <c r="M21" s="4" t="inlineStr">
@@ -3334,7 +3340,7 @@
       </c>
       <c r="N21" s="4" t="inlineStr">
         <is>
-          <t>Pickup : 2026-09-08, Return : 2026-09-11</t>
+          <t>Pickup : 2026-09-08, Return : 2026-09-14 / FIRST DATE CAN RETURN CNTR DD.14/09 WITHOUT RENT</t>
         </is>
       </c>
       <c r="O21" s="4" t="n">
@@ -3344,7 +3350,7 @@
         <v>0</v>
       </c>
       <c r="Q21" s="4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="R21" s="4" t="n">
         <v>0</v>
@@ -3412,249 +3418,108 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>HASLS22260900696</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="inlineStr">
-        <is>
-          <t>SWAL</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
-        <is>
-          <t>2608N</t>
-        </is>
-      </c>
-      <c r="D22" s="4" t="inlineStr">
-        <is>
-          <t>202609281500</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="inlineStr"/>
-      <c r="F22" s="4" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H22" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40Hx1 </t>
-        </is>
-      </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>20260825</t>
-        </is>
-      </c>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>FREIGHT LINKS EXPRESS (THAILAND) CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>FEDERAL-MOGUL (THAILAND) COMPANY LIMITED</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>EMPTY PLASTIC BOBBIN</t>
-        </is>
-      </c>
-      <c r="M22" s="4" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="N22" s="4" t="inlineStr">
-        <is>
-          <t>Pickup : 2026-08-25, Return : 2026-08-26</t>
-        </is>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="R22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Y22" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z22" s="4">
-        <f>SUM(O22:W22)-X22</f>
-        <v/>
-      </c>
-      <c r="AA22" s="4">
-        <f>MAX(0,O22-MAX(0,X22))</f>
-        <v/>
-      </c>
-      <c r="AB22" s="4">
-        <f>MAX(0,P22-MAX(0,X22-SUM(O22:O22)))</f>
-        <v/>
-      </c>
-      <c r="AC22" s="4">
-        <f>MAX(0,Q22-MAX(0,X22-SUM(O22:P22)))</f>
-        <v/>
-      </c>
-      <c r="AD22" s="4">
-        <f>MAX(0,R22-MAX(0,X22-SUM(O22:Q22)))</f>
-        <v/>
-      </c>
-      <c r="AE22" s="4">
-        <f>MAX(0,S22-MAX(0,X22-SUM(O22:R22)))</f>
-        <v/>
-      </c>
-      <c r="AF22" s="4">
-        <f>MAX(0,T22-MAX(0,X22-SUM(O22:S22)))</f>
-        <v/>
-      </c>
-      <c r="AG22" s="4">
-        <f>MAX(0,U22-MAX(0,X22-SUM(O22:T22)))</f>
-        <v/>
-      </c>
-      <c r="AH22" s="4">
-        <f>MAX(0,V22-MAX(0,X22-SUM(O22:U22)))</f>
-        <v/>
-      </c>
-      <c r="AI22" s="4">
-        <f>MAX(0,W22-MAX(0,X22-SUM(O22:V22)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A22" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B23" s="5" t="n"/>
-      <c r="C23" s="5" t="n"/>
-      <c r="D23" s="5" t="n"/>
-      <c r="E23" s="5" t="n"/>
-      <c r="F23" s="5" t="n"/>
-      <c r="G23" s="5" t="n"/>
-      <c r="H23" s="5" t="n"/>
-      <c r="I23" s="5" t="n"/>
-      <c r="J23" s="5" t="n"/>
-      <c r="K23" s="5" t="n"/>
-      <c r="L23" s="5" t="n"/>
-      <c r="M23" s="5" t="n"/>
-      <c r="N23" s="5" t="n"/>
-      <c r="O23" s="5">
-        <f>SUM(O3:O22)</f>
-        <v/>
-      </c>
-      <c r="P23" s="5">
-        <f>SUM(P3:P22)</f>
-        <v/>
-      </c>
-      <c r="Q23" s="5">
-        <f>SUM(Q3:Q22)</f>
-        <v/>
-      </c>
-      <c r="R23" s="5">
-        <f>SUM(R3:R22)</f>
-        <v/>
-      </c>
-      <c r="S23" s="5">
-        <f>SUM(S3:S22)</f>
-        <v/>
-      </c>
-      <c r="T23" s="5">
-        <f>SUM(T3:T22)</f>
-        <v/>
-      </c>
-      <c r="U23" s="5">
-        <f>SUM(U3:U22)</f>
-        <v/>
-      </c>
-      <c r="V23" s="5">
-        <f>SUM(V3:V22)</f>
-        <v/>
-      </c>
-      <c r="W23" s="5">
-        <f>SUM(W3:W22)</f>
-        <v/>
-      </c>
-      <c r="X23" s="5">
-        <f>SUM(X3:X22)</f>
-        <v/>
-      </c>
-      <c r="Y23" s="5" t="n"/>
-      <c r="Z23" s="5">
-        <f>SUM(Z3:Z22)</f>
-        <v/>
-      </c>
-      <c r="AA23" s="5">
-        <f>SUM(AA3:AA22)</f>
-        <v/>
-      </c>
-      <c r="AB23" s="5">
-        <f>SUM(AB3:AB22)</f>
-        <v/>
-      </c>
-      <c r="AC23" s="5">
-        <f>SUM(AC3:AC22)</f>
-        <v/>
-      </c>
-      <c r="AD23" s="5">
-        <f>SUM(AD3:AD22)</f>
-        <v/>
-      </c>
-      <c r="AE23" s="5">
-        <f>SUM(AE3:AE22)</f>
-        <v/>
-      </c>
-      <c r="AF23" s="5">
-        <f>SUM(AF3:AF22)</f>
-        <v/>
-      </c>
-      <c r="AG23" s="5">
-        <f>SUM(AG3:AG22)</f>
-        <v/>
-      </c>
-      <c r="AH23" s="5">
-        <f>SUM(AH3:AH22)</f>
-        <v/>
-      </c>
-      <c r="AI23" s="5">
-        <f>SUM(AI3:AI22)</f>
+      <c r="B22" s="5" t="n"/>
+      <c r="C22" s="5" t="n"/>
+      <c r="D22" s="5" t="n"/>
+      <c r="E22" s="5" t="n"/>
+      <c r="F22" s="5" t="n"/>
+      <c r="G22" s="5" t="n"/>
+      <c r="H22" s="5" t="n"/>
+      <c r="I22" s="5" t="n"/>
+      <c r="J22" s="5" t="n"/>
+      <c r="K22" s="5" t="n"/>
+      <c r="L22" s="5" t="n"/>
+      <c r="M22" s="5" t="n"/>
+      <c r="N22" s="5" t="n"/>
+      <c r="O22" s="5">
+        <f>SUM(O3:O21)</f>
+        <v/>
+      </c>
+      <c r="P22" s="5">
+        <f>SUM(P3:P21)</f>
+        <v/>
+      </c>
+      <c r="Q22" s="5">
+        <f>SUM(Q3:Q21)</f>
+        <v/>
+      </c>
+      <c r="R22" s="5">
+        <f>SUM(R3:R21)</f>
+        <v/>
+      </c>
+      <c r="S22" s="5">
+        <f>SUM(S3:S21)</f>
+        <v/>
+      </c>
+      <c r="T22" s="5">
+        <f>SUM(T3:T21)</f>
+        <v/>
+      </c>
+      <c r="U22" s="5">
+        <f>SUM(U3:U21)</f>
+        <v/>
+      </c>
+      <c r="V22" s="5">
+        <f>SUM(V3:V21)</f>
+        <v/>
+      </c>
+      <c r="W22" s="5">
+        <f>SUM(W3:W21)</f>
+        <v/>
+      </c>
+      <c r="X22" s="5">
+        <f>SUM(X3:X21)</f>
+        <v/>
+      </c>
+      <c r="Y22" s="5" t="n"/>
+      <c r="Z22" s="5">
+        <f>SUM(Z3:Z21)</f>
+        <v/>
+      </c>
+      <c r="AA22" s="5">
+        <f>SUM(AA3:AA21)</f>
+        <v/>
+      </c>
+      <c r="AB22" s="5">
+        <f>SUM(AB3:AB21)</f>
+        <v/>
+      </c>
+      <c r="AC22" s="5">
+        <f>SUM(AC3:AC21)</f>
+        <v/>
+      </c>
+      <c r="AD22" s="5">
+        <f>SUM(AD3:AD21)</f>
+        <v/>
+      </c>
+      <c r="AE22" s="5">
+        <f>SUM(AE3:AE21)</f>
+        <v/>
+      </c>
+      <c r="AF22" s="5">
+        <f>SUM(AF3:AF21)</f>
+        <v/>
+      </c>
+      <c r="AG22" s="5">
+        <f>SUM(AG3:AG21)</f>
+        <v/>
+      </c>
+      <c r="AH22" s="5">
+        <f>SUM(AH3:AH21)</f>
+        <v/>
+      </c>
+      <c r="AI22" s="5">
+        <f>SUM(AI3:AI21)</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AI22"/>
+  <autoFilter ref="A2:AI21"/>
   <mergeCells count="1">
     <mergeCell ref="A1:AI1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Update dashboard and reports with 9-16-PD booking data
Regenerated from "9-16-PD.xls" (2710 rows): 117 BK No outstanding,
269 containers. HASLS22260900416 is still flagged for missing
Pickup Name — now unresolved for 5 consecutive days of data.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - B.C. DEPOT CO.,LTD. ( Bang-Na KM.18).xlsx
+++ b/output/bkg pending - B.C. DEPOT CO.,LTD. ( Bang-Na KM.18).xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$2:$AG$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$2:$AG$26</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -484,7 +484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG36"/>
+  <dimension ref="A1:AG32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -746,10 +746,10 @@
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>202609211300</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="n"/>
+          <t>202609210900</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr"/>
       <c r="F3" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -862,25 +862,25 @@
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801247</t>
+          <t>HASLS22260801252</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>PGPO</t>
+          <t>KJT</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>202609221600</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="n"/>
+          <t>202609222100</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr"/>
       <c r="F4" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -888,42 +888,42 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>KRPUS</t>
+          <t>HKHKG</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx4 </t>
+          <t xml:space="preserve">20'x4 </t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>20260915</t>
+          <t>20260910</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>NEOCOSMED CO., LTD.</t>
+          <t>CHEVRON (THAILAND) LIMITED</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>TOOTHPASTE</t>
+          <t>LUBE OIL</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>Req. Container condition  GRADE B+ CNTR / CLEAN CNTR WITH GOOD CONDITION / NO SMELL/NODAMAGES / STRONG &amp; SMOOTH FLOOR / NO NAILS / LOAD UNDERDECK</t>
         </is>
       </c>
       <c r="M4" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>0</v>
@@ -944,7 +944,7 @@
         <v>0</v>
       </c>
       <c r="V4" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W4" s="4" t="n">
         <v>0</v>
@@ -993,12 +993,12 @@
     <row r="5" ht="13" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801252</t>
+          <t>HASLS22260801423</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>KJT</t>
+          <t>KMGY</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
@@ -1008,10 +1008,10 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>202609220800</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="n"/>
+          <t>202609271700</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr"/>
       <c r="F5" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -1019,36 +1019,36 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>CNXMN</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x4 </t>
+          <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>20260910</t>
+          <t>20260915</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>CHEVRON (THAILAND) LIMITED</t>
+          <t>TAKO FOODS INDUSTRY CO., LTD.</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>LUBE OIL</t>
+          <t>COCONUT WATER</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Req. Container condition  GRADE B+ CNTR / CLEAN CNTR WITH GOOD CONDITION / NO SMELL/NODAMAGES / STRONG &amp; SMOOTH FLOOR / NO NAILS / LOAD UNDERDECK</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M5" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N5" s="4" t="n">
         <v>0</v>
@@ -1075,7 +1075,7 @@
         <v>0</v>
       </c>
       <c r="V5" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="W5" s="4" t="n">
         <v>0</v>
@@ -1124,62 +1124,66 @@
     <row r="6" ht="13" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801423</t>
+          <t>HASLS22260801587</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>KMGY</t>
+          <t>NSSJ</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2607S</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>202609271700</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="n"/>
+          <t>202609220800</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>THLKR</t>
+        </is>
+      </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>CNXMN</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>20260915</t>
+          <t>20260912</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>TAKO FOODS INDUSTRY CO., LTD.</t>
+          <t>MEDIFOODS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>COCONUT WATER</t>
+          <t>ORGANIC JASMINE RICE FLOUR 120MESH</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>GOOD &amp; CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M6" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>0</v>
@@ -1255,66 +1259,63 @@
     <row r="7" ht="13" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801587</t>
+          <t>HASLS22260801914</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>NSSJ</t>
+          <t>SWMM</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>2607S</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>202609220800</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>THLKR</t>
-        </is>
-      </c>
+          <t>202609230900</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr"/>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>THLCH</t>
+          <t>THBKK</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>IDJKT</t>
+          <t>KRPTK</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">20'x33 </t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
         <is>
-          <t>20260912</t>
+          <t>20260915</t>
         </is>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>MEDIFOODS (THAILAND) CO., LTD.</t>
+          <t>DP WORLD LOGISTICS SOLUTIONS (THAILAND) COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>ORGANIC JASMINE RICE FLOUR 120MESH</t>
+          <t>SOYBEAN OIL</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>GOOD &amp; CLEAN CONTAINER</t>
+          <t>** APPROVAL MR.KIM GEON WOOK DD.25/08/2026  ** *FLEXIBAG ONDECK*
+Servey: 15/09/2026, Pickup : 16/09/2026</t>
         </is>
       </c>
       <c r="M7" s="4" t="n">
-        <v>1</v>
+        <v>33</v>
       </c>
       <c r="N7" s="4" t="n">
         <v>0</v>
@@ -1390,25 +1391,25 @@
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801612</t>
+          <t>HASLS22260801939</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>CMA</t>
+          <t>SWSP</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>2614N</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>202609241200</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="n"/>
+          <t>202610022300</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr"/>
       <c r="F8" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -1416,36 +1417,36 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">20'x7 </t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>20260908</t>
+          <t>20260907</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>DUNI (THAILAND) CO., LTD.</t>
+          <t>THAI GYPSUM PRODUCTS PCL.</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PAPER NAPKIN </t>
+          <t>GYPSUM PLASTER - 25202090</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>REQ. GOOD GRADE CONTAINER</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M8" s="4" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>0</v>
@@ -1521,25 +1522,25 @@
     <row r="9" ht="13" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801626</t>
+          <t>HASLS22260802080</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>KMTP</t>
+          <t>SWIC</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>202609200900</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="n"/>
+          <t>202609211200</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr"/>
       <c r="F9" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -1547,36 +1548,36 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">20'x14 </t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>20260915</t>
+          <t>20260916</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>THAI ASIA METAL AND TECHNO INDUSTRY CO., LTD.</t>
+          <t>THAI FERMENTATION INDUSTRY CO., LTD.</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>PIPE</t>
+          <t>MSG</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>GOOD &amp; CLEAN CONT. NO SMELL</t>
+          <t>REQ food grate ctn</t>
         </is>
       </c>
       <c r="M9" s="4" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="N9" s="4" t="n">
         <v>0</v>
@@ -1603,7 +1604,7 @@
         <v>0</v>
       </c>
       <c r="V9" s="4" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="W9" s="4" t="n">
         <v>0</v>
@@ -1652,25 +1653,25 @@
     <row r="10" ht="13" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801726</t>
+          <t>HASLS22260802148</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>PGPO</t>
+          <t>KJT</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>202609221600</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="n"/>
+          <t>202609222100</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr"/>
       <c r="F10" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -1678,42 +1679,42 @@
       </c>
       <c r="G10" s="4" t="inlineStr">
         <is>
-          <t>KRKAN</t>
+          <t>HKHKG</t>
         </is>
       </c>
       <c r="H10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
         <is>
-          <t>20260912</t>
+          <t>20260916</t>
         </is>
       </c>
       <c r="J10" s="4" t="inlineStr">
         <is>
-          <t>THAI ASAHI CO., LTD.</t>
+          <t>SINGHA WORLDWIDE INTERNATIONAL CO., LTD.</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">POTATO STARCH </t>
+          <t>SODA WATER</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Grade A and food grade container</t>
+          <t>Under desk cargo and food grade container</t>
         </is>
       </c>
       <c r="M10" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N10" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O10" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P10" s="4" t="n">
         <v>0</v>
@@ -1781,527 +1782,526 @@
       </c>
     </row>
     <row r="11" ht="13" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>HASLS22260801774</t>
-        </is>
-      </c>
-      <c r="B11" s="4" t="inlineStr">
-        <is>
-          <t>KMTP</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>2611N</t>
-        </is>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>202609200900</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="n"/>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>HASLS22260802265</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>CMA</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>2614N</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>202609241200</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr"/>
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>CNXMN</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40Hx4 </t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>20260915</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>COSMOS BREWERY (THAILAND) CO.,LTD.</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>CHANG SODA WATER</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>RQST GOOD CLEAN &amp; DRY CONT.</t>
-        </is>
-      </c>
-      <c r="M11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="P11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V11" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="W11" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X11" s="4">
+      <c r="G11" s="5" t="inlineStr">
+        <is>
+          <t>HKHKG</t>
+        </is>
+      </c>
+      <c r="H11" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R40Hx1 </t>
+        </is>
+      </c>
+      <c r="I11" s="5" t="inlineStr">
+        <is>
+          <t>20260914</t>
+        </is>
+      </c>
+      <c r="J11" s="5" t="inlineStr">
+        <is>
+          <t>KIBUN (THAILAND) CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K11" s="5" t="inlineStr">
+        <is>
+          <t>FROZEN IMITATION CRAB MEAT</t>
+        </is>
+      </c>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>(Temp -20.0 / Vent Close)  **REQ GOOD, CLEAN, NO LEAK AND GRADE A CONTAINER</t>
+        </is>
+      </c>
+      <c r="M11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="R11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X11" s="5">
         <f>SUM(M11:U11)-V11</f>
         <v/>
       </c>
-      <c r="Y11" s="4">
+      <c r="Y11" s="5">
         <f>MAX(0,M11-MAX(0,V11))</f>
         <v/>
       </c>
-      <c r="Z11" s="4">
+      <c r="Z11" s="5">
         <f>MAX(0,N11-MAX(0,V11-SUM(M11:M11)))</f>
         <v/>
       </c>
-      <c r="AA11" s="4">
+      <c r="AA11" s="5">
         <f>MAX(0,O11-MAX(0,V11-SUM(M11:N11)))</f>
         <v/>
       </c>
-      <c r="AB11" s="4">
+      <c r="AB11" s="5">
         <f>MAX(0,P11-MAX(0,V11-SUM(M11:O11)))</f>
         <v/>
       </c>
-      <c r="AC11" s="4">
+      <c r="AC11" s="5">
         <f>MAX(0,Q11-MAX(0,V11-SUM(M11:P11)))</f>
         <v/>
       </c>
-      <c r="AD11" s="4">
+      <c r="AD11" s="5">
         <f>MAX(0,R11-MAX(0,V11-SUM(M11:Q11)))</f>
         <v/>
       </c>
-      <c r="AE11" s="4">
+      <c r="AE11" s="5">
         <f>MAX(0,S11-MAX(0,V11-SUM(M11:R11)))</f>
         <v/>
       </c>
-      <c r="AF11" s="4">
+      <c r="AF11" s="5">
         <f>MAX(0,T11-MAX(0,V11-SUM(M11:S11)))</f>
         <v/>
       </c>
-      <c r="AG11" s="4">
+      <c r="AG11" s="5">
         <f>MAX(0,U11-MAX(0,V11-SUM(M11:T11)))</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="13" customHeight="1">
-      <c r="A12" s="4" t="inlineStr">
-        <is>
-          <t>HASLS22260801815</t>
-        </is>
-      </c>
-      <c r="B12" s="4" t="inlineStr">
-        <is>
-          <t>SWBT</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
-        <is>
-          <t>2615N</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>202609211300</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="n"/>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>HASLS22260802566</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>SWAT</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>2611N</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>202610251024</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr"/>
+      <c r="F12" s="5" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G12" s="4" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H12" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x2 </t>
-        </is>
-      </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>20260915</t>
-        </is>
-      </c>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>THANAKORN VEGETABLE OIL PRODUCTS CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>LECITHIN</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>** APPROVED BY GHL DD.25/08/2026** *FLEXIBAG ONDECK*
-Survey : 2026-09-15, Pickup : 2026-09-16 REQUEST STRONG, CLEAN, FOOD GRADE CONTAINER</t>
-        </is>
-      </c>
-      <c r="M12" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="N12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W12" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X12" s="4">
+      <c r="G12" s="5" t="inlineStr">
+        <is>
+          <t>KRPUS</t>
+        </is>
+      </c>
+      <c r="H12" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R40Hx1 </t>
+        </is>
+      </c>
+      <c r="I12" s="5" t="inlineStr">
+        <is>
+          <t>20260916</t>
+        </is>
+      </c>
+      <c r="J12" s="5" t="inlineStr">
+        <is>
+          <t>N&amp;N FOODS CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K12" s="5" t="inlineStr">
+        <is>
+          <t>FROZEN FOOD</t>
+        </is>
+      </c>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>(Temp -20.0℃ / Vent Close) Request good and clean container</t>
+        </is>
+      </c>
+      <c r="M12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="R12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X12" s="5">
         <f>SUM(M12:U12)-V12</f>
         <v/>
       </c>
-      <c r="Y12" s="4">
+      <c r="Y12" s="5">
         <f>MAX(0,M12-MAX(0,V12))</f>
         <v/>
       </c>
-      <c r="Z12" s="4">
+      <c r="Z12" s="5">
         <f>MAX(0,N12-MAX(0,V12-SUM(M12:M12)))</f>
         <v/>
       </c>
-      <c r="AA12" s="4">
+      <c r="AA12" s="5">
         <f>MAX(0,O12-MAX(0,V12-SUM(M12:N12)))</f>
         <v/>
       </c>
-      <c r="AB12" s="4">
+      <c r="AB12" s="5">
         <f>MAX(0,P12-MAX(0,V12-SUM(M12:O12)))</f>
         <v/>
       </c>
-      <c r="AC12" s="4">
+      <c r="AC12" s="5">
         <f>MAX(0,Q12-MAX(0,V12-SUM(M12:P12)))</f>
         <v/>
       </c>
-      <c r="AD12" s="4">
+      <c r="AD12" s="5">
         <f>MAX(0,R12-MAX(0,V12-SUM(M12:Q12)))</f>
         <v/>
       </c>
-      <c r="AE12" s="4">
+      <c r="AE12" s="5">
         <f>MAX(0,S12-MAX(0,V12-SUM(M12:R12)))</f>
         <v/>
       </c>
-      <c r="AF12" s="4">
+      <c r="AF12" s="5">
         <f>MAX(0,T12-MAX(0,V12-SUM(M12:S12)))</f>
         <v/>
       </c>
-      <c r="AG12" s="4">
+      <c r="AG12" s="5">
         <f>MAX(0,U12-MAX(0,V12-SUM(M12:T12)))</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="13" customHeight="1">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>HASLS22260801914</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>SWMM</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>2609N</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>202609230900</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="n"/>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>HASLS22260802575</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>SWIC</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>202609211200</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr"/>
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>KRPTK</t>
-        </is>
-      </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x33 </t>
-        </is>
-      </c>
-      <c r="I13" s="4" t="inlineStr">
-        <is>
-          <t>20260915</t>
-        </is>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>DP WORLD LOGISTICS SOLUTIONS (THAILAND) COMPANY LIMITED</t>
-        </is>
-      </c>
-      <c r="K13" s="4" t="inlineStr">
-        <is>
-          <t>SOYBEAN OIL</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>** APPROVAL MR.KIM GEON WOOK DD.25/08/2026  ** *FLEXIBAG ONDECK*
-Servey: 15/09/2026, Pickup : 16/09/2026</t>
-        </is>
-      </c>
-      <c r="M13" s="4" t="n">
-        <v>33</v>
-      </c>
-      <c r="N13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W13" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X13" s="4">
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R40Hx6 </t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>20260914</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>GOLDEN PRIZE CANNING CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>FROZEN TUNA</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>(Temp -25.0℃ / Vent Close)
+REQUEST GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="R13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V13" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="W13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" s="5">
         <f>SUM(M13:U13)-V13</f>
         <v/>
       </c>
-      <c r="Y13" s="4">
+      <c r="Y13" s="5">
         <f>MAX(0,M13-MAX(0,V13))</f>
         <v/>
       </c>
-      <c r="Z13" s="4">
+      <c r="Z13" s="5">
         <f>MAX(0,N13-MAX(0,V13-SUM(M13:M13)))</f>
         <v/>
       </c>
-      <c r="AA13" s="4">
+      <c r="AA13" s="5">
         <f>MAX(0,O13-MAX(0,V13-SUM(M13:N13)))</f>
         <v/>
       </c>
-      <c r="AB13" s="4">
+      <c r="AB13" s="5">
         <f>MAX(0,P13-MAX(0,V13-SUM(M13:O13)))</f>
         <v/>
       </c>
-      <c r="AC13" s="4">
+      <c r="AC13" s="5">
         <f>MAX(0,Q13-MAX(0,V13-SUM(M13:P13)))</f>
         <v/>
       </c>
-      <c r="AD13" s="4">
+      <c r="AD13" s="5">
         <f>MAX(0,R13-MAX(0,V13-SUM(M13:Q13)))</f>
         <v/>
       </c>
-      <c r="AE13" s="4">
+      <c r="AE13" s="5">
         <f>MAX(0,S13-MAX(0,V13-SUM(M13:R13)))</f>
         <v/>
       </c>
-      <c r="AF13" s="4">
+      <c r="AF13" s="5">
         <f>MAX(0,T13-MAX(0,V13-SUM(M13:S13)))</f>
         <v/>
       </c>
-      <c r="AG13" s="4">
+      <c r="AG13" s="5">
         <f>MAX(0,U13-MAX(0,V13-SUM(M13:T13)))</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="13" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>HASLS22260801939</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>SWBT</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>HASLS22260900037</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>KUS</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>2615N</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>202609211300</t>
-        </is>
-      </c>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>202609222100</t>
+        </is>
+      </c>
+      <c r="E14" s="5" t="inlineStr"/>
+      <c r="F14" s="5" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="5" t="inlineStr">
         <is>
           <t>VNSGN</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40Hx1 </t>
-        </is>
-      </c>
-      <c r="I14" s="4" t="inlineStr">
-        <is>
-          <t>20260905</t>
-        </is>
-      </c>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>VISTA DISTRIBUTION CO.,LTD.</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>SNACK</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="4" t="n">
+      <c r="H14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R40Hx2 </t>
+        </is>
+      </c>
+      <c r="I14" s="5" t="inlineStr">
+        <is>
+          <t>20260916</t>
+        </is>
+      </c>
+      <c r="J14" s="5" t="inlineStr">
+        <is>
+          <t>INVE (THAILAND) LTD</t>
+        </is>
+      </c>
+      <c r="K14" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ANIMAL FEED </t>
+        </is>
+      </c>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>(Temp +2.0℃ / Vent Close) REQUEST GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="R14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V14" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="P14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W14" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X14" s="4">
+      <c r="W14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X14" s="5">
         <f>SUM(M14:U14)-V14</f>
         <v/>
       </c>
-      <c r="Y14" s="4">
+      <c r="Y14" s="5">
         <f>MAX(0,M14-MAX(0,V14))</f>
         <v/>
       </c>
-      <c r="Z14" s="4">
+      <c r="Z14" s="5">
         <f>MAX(0,N14-MAX(0,V14-SUM(M14:M14)))</f>
         <v/>
       </c>
-      <c r="AA14" s="4">
+      <c r="AA14" s="5">
         <f>MAX(0,O14-MAX(0,V14-SUM(M14:N14)))</f>
         <v/>
       </c>
-      <c r="AB14" s="4">
+      <c r="AB14" s="5">
         <f>MAX(0,P14-MAX(0,V14-SUM(M14:O14)))</f>
         <v/>
       </c>
-      <c r="AC14" s="4">
+      <c r="AC14" s="5">
         <f>MAX(0,Q14-MAX(0,V14-SUM(M14:P14)))</f>
         <v/>
       </c>
-      <c r="AD14" s="4">
+      <c r="AD14" s="5">
         <f>MAX(0,R14-MAX(0,V14-SUM(M14:Q14)))</f>
         <v/>
       </c>
-      <c r="AE14" s="4">
+      <c r="AE14" s="5">
         <f>MAX(0,S14-MAX(0,V14-SUM(M14:R14)))</f>
         <v/>
       </c>
-      <c r="AF14" s="4">
+      <c r="AF14" s="5">
         <f>MAX(0,T14-MAX(0,V14-SUM(M14:S14)))</f>
         <v/>
       </c>
-      <c r="AG14" s="4">
+      <c r="AG14" s="5">
         <f>MAX(0,U14-MAX(0,V14-SUM(M14:T14)))</f>
         <v/>
       </c>
@@ -2309,25 +2309,25 @@
     <row r="15" ht="13" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260802240</t>
+          <t>HASLS22260900089</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>KMTP</t>
+          <t>SWIC</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>202609200900</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="n"/>
+          <t>202609211200</t>
+        </is>
+      </c>
+      <c r="E15" s="4" t="inlineStr"/>
       <c r="F15" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -2335,27 +2335,27 @@
       </c>
       <c r="G15" s="4" t="inlineStr">
         <is>
-          <t>CNXMN</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x6 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I15" s="4" t="inlineStr">
         <is>
-          <t>20260912</t>
+          <t>20260915</t>
         </is>
       </c>
       <c r="J15" s="4" t="inlineStr">
         <is>
-          <t>STARPRO STARCH (THAILAND) CO., LTD.</t>
+          <t>SITTHINAN CO., LTD.</t>
         </is>
       </c>
       <c r="K15" s="4" t="inlineStr">
         <is>
-          <t>STARCH</t>
+          <t>MUNG BEAN STARCH</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
@@ -2364,7 +2364,7 @@
         </is>
       </c>
       <c r="M15" s="4" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N15" s="4" t="n">
         <v>0</v>
@@ -2438,132 +2438,132 @@
       </c>
     </row>
     <row r="16" ht="13" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>HASLS22260802265</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>CMA</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>2614N</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>202609241200</t>
-        </is>
-      </c>
-      <c r="E16" s="5" t="n"/>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260900295</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>KJT</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>202609222100</t>
+        </is>
+      </c>
+      <c r="E16" s="4" t="inlineStr"/>
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
-        <is>
-          <t>HKHKG</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R40Hx1 </t>
-        </is>
-      </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>TWKEL</t>
+        </is>
+      </c>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>20260914</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
-        <is>
-          <t>KIBUN (THAILAND) CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K16" s="5" t="inlineStr">
-        <is>
-          <t>FROZEN IMITATION CRAB MEAT</t>
-        </is>
-      </c>
-      <c r="L16" s="5" t="inlineStr">
-        <is>
-          <t>(Temp -20.0 / Vent Close)  **REQ GOOD, CLEAN, NO LEAK AND GRADE A CONTAINER</t>
-        </is>
-      </c>
-      <c r="M16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="5" t="n">
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>DZQ CO.,LTD.</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>FOODSTUFFS</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>CONTAINER GOOD AND CLEAN</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X16" s="5">
+      <c r="N16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X16" s="4">
         <f>SUM(M16:U16)-V16</f>
         <v/>
       </c>
-      <c r="Y16" s="5">
+      <c r="Y16" s="4">
         <f>MAX(0,M16-MAX(0,V16))</f>
         <v/>
       </c>
-      <c r="Z16" s="5">
+      <c r="Z16" s="4">
         <f>MAX(0,N16-MAX(0,V16-SUM(M16:M16)))</f>
         <v/>
       </c>
-      <c r="AA16" s="5">
+      <c r="AA16" s="4">
         <f>MAX(0,O16-MAX(0,V16-SUM(M16:N16)))</f>
         <v/>
       </c>
-      <c r="AB16" s="5">
+      <c r="AB16" s="4">
         <f>MAX(0,P16-MAX(0,V16-SUM(M16:O16)))</f>
         <v/>
       </c>
-      <c r="AC16" s="5">
+      <c r="AC16" s="4">
         <f>MAX(0,Q16-MAX(0,V16-SUM(M16:P16)))</f>
         <v/>
       </c>
-      <c r="AD16" s="5">
+      <c r="AD16" s="4">
         <f>MAX(0,R16-MAX(0,V16-SUM(M16:Q16)))</f>
         <v/>
       </c>
-      <c r="AE16" s="5">
+      <c r="AE16" s="4">
         <f>MAX(0,S16-MAX(0,V16-SUM(M16:R16)))</f>
         <v/>
       </c>
-      <c r="AF16" s="5">
+      <c r="AF16" s="4">
         <f>MAX(0,T16-MAX(0,V16-SUM(M16:S16)))</f>
         <v/>
       </c>
-      <c r="AG16" s="5">
+      <c r="AG16" s="4">
         <f>MAX(0,U16-MAX(0,V16-SUM(M16:T16)))</f>
         <v/>
       </c>
@@ -2571,68 +2571,72 @@
     <row r="17" ht="13" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260802380</t>
+          <t>HASLS22260900311</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>KUS</t>
+          <t>HAB</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>2615N</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>202609222100</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="n"/>
+          <t>202609270600</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>THSRP</t>
+        </is>
+      </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>KRINC</t>
+          <t>CNSHA</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>20260903</t>
+          <t>20260915</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>ASIAN FOODS CO.,LTD.</t>
+          <t>SMS CORPORATION CO., LTD.</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">KRISPY ROLL </t>
+          <t>MODIFIED TAPIOCA STARCH</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>FOOD GRADE CONTAINER / DO NOT RELEASE RED WALL CONTAINER</t>
         </is>
       </c>
       <c r="M17" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N17" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O17" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P17" s="4" t="n">
         <v>0</v>
@@ -2702,25 +2706,25 @@
     <row r="18" ht="13" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260802434</t>
+          <t>HASLS22260900552</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>SWBT</t>
+          <t>KJT</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>2615N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>202609211300</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="n"/>
+          <t>202609222100</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr"/>
       <c r="F18" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -2728,32 +2732,32 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>CNSHK</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">40Hx2 </t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>20260914</t>
+          <t>20260916</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>TNA INTERNATIONAL CO.,LTD.</t>
+          <t>NMB-MINEBEA THAI LTD.</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>FERTILIZER</t>
+          <t>BALL BEARING</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>RQS CLEAN &amp; GOOD CONTAINER CONDITION.</t>
+          <t>REQUEST CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M18" s="4" t="n">
@@ -2763,7 +2767,7 @@
         <v>0</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P18" s="4" t="n">
         <v>0</v>
@@ -2833,25 +2837,25 @@
     <row r="19" ht="13" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>HASLS22260802575</t>
+          <t>HASLS22260900747</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>SWIC</t>
+          <t>SWBT</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2615N</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>202609211000</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="n"/>
+          <t>202609210900</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr"/>
       <c r="F19" s="5" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -2864,28 +2868,27 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">R40Hx6 </t>
+          <t xml:space="preserve">R40Hx1 </t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>20260914</t>
+          <t>20260916</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>GOLDEN PRIZE CANNING CO., LTD.</t>
+          <t>MEGA LIFESCIENCES PUBLIC CO., LTD.</t>
         </is>
       </c>
       <c r="K19" s="5" t="inlineStr">
         <is>
-          <t>FROZEN TUNA</t>
+          <t>PHARMACEUTICAL PRODUCTS</t>
         </is>
       </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
-          <t>(Temp -25.0℃ / Vent Close)
-REQUEST GOOD AND CLEAN CONTAINER</t>
+          <t>Temp  +22.0℃ / Vent Close)</t>
         </is>
       </c>
       <c r="M19" s="5" t="n">
@@ -2901,7 +2904,7 @@
         <v>0</v>
       </c>
       <c r="Q19" s="5" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="R19" s="5" t="n">
         <v>0</v>
@@ -2916,7 +2919,7 @@
         <v>0</v>
       </c>
       <c r="V19" s="5" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="W19" s="5" t="n">
         <v>0</v>
@@ -2963,132 +2966,132 @@
       </c>
     </row>
     <row r="20" ht="13" customHeight="1">
-      <c r="A20" s="4" t="inlineStr">
-        <is>
-          <t>HASLS22260900005</t>
-        </is>
-      </c>
-      <c r="B20" s="4" t="inlineStr">
-        <is>
-          <t>SWIC</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
-        <is>
-          <t>2610N</t>
-        </is>
-      </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>202609211000</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="n"/>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>HASLS22260900748</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>SWBT</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>2615N</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>202609210900</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr"/>
+      <c r="F20" s="5" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G20" s="5" t="inlineStr">
         <is>
           <t>VNSGN</t>
         </is>
       </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I20" s="4" t="inlineStr">
-        <is>
-          <t>20260915</t>
-        </is>
-      </c>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
-          <t>ASAHIKASEI PLASTICS (THAILAND) CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>POLYAMIDE PLASTIC PELLET</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M20" s="4" t="n">
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R40Hx1 </t>
+        </is>
+      </c>
+      <c r="I20" s="5" t="inlineStr">
+        <is>
+          <t>20260916</t>
+        </is>
+      </c>
+      <c r="J20" s="5" t="inlineStr">
+        <is>
+          <t>MEGA LIFESCIENCES PUBLIC CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K20" s="5" t="inlineStr">
+        <is>
+          <t>PHARMACEUTICAL PRODUCTS</t>
+        </is>
+      </c>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>(Temp +22.0℃ / Vent Close)</t>
+        </is>
+      </c>
+      <c r="M20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="N20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W20" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X20" s="4">
+      <c r="R20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="V20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="W20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X20" s="5">
         <f>SUM(M20:U20)-V20</f>
         <v/>
       </c>
-      <c r="Y20" s="4">
+      <c r="Y20" s="5">
         <f>MAX(0,M20-MAX(0,V20))</f>
         <v/>
       </c>
-      <c r="Z20" s="4">
+      <c r="Z20" s="5">
         <f>MAX(0,N20-MAX(0,V20-SUM(M20:M20)))</f>
         <v/>
       </c>
-      <c r="AA20" s="4">
+      <c r="AA20" s="5">
         <f>MAX(0,O20-MAX(0,V20-SUM(M20:N20)))</f>
         <v/>
       </c>
-      <c r="AB20" s="4">
+      <c r="AB20" s="5">
         <f>MAX(0,P20-MAX(0,V20-SUM(M20:O20)))</f>
         <v/>
       </c>
-      <c r="AC20" s="4">
+      <c r="AC20" s="5">
         <f>MAX(0,Q20-MAX(0,V20-SUM(M20:P20)))</f>
         <v/>
       </c>
-      <c r="AD20" s="4">
+      <c r="AD20" s="5">
         <f>MAX(0,R20-MAX(0,V20-SUM(M20:Q20)))</f>
         <v/>
       </c>
-      <c r="AE20" s="4">
+      <c r="AE20" s="5">
         <f>MAX(0,S20-MAX(0,V20-SUM(M20:R20)))</f>
         <v/>
       </c>
-      <c r="AF20" s="4">
+      <c r="AF20" s="5">
         <f>MAX(0,T20-MAX(0,V20-SUM(M20:S20)))</f>
         <v/>
       </c>
-      <c r="AG20" s="4">
+      <c r="AG20" s="5">
         <f>MAX(0,U20-MAX(0,V20-SUM(M20:T20)))</f>
         <v/>
       </c>
@@ -3096,25 +3099,25 @@
     <row r="21" ht="13" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260900075</t>
+          <t>HASLS22260900775</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>KMTP</t>
+          <t>SWDN</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>202609200900</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="n"/>
+          <t>202609300900</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr"/>
       <c r="F21" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -3122,7 +3125,7 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>KRINC</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
@@ -3132,22 +3135,22 @@
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>20260914</t>
+          <t>20260915</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>J &amp; B SIAM MARKETING CO.,LTD.</t>
+          <t>I-TAIL CORPORATION PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">FOODSTUFFS </t>
+          <t>PET FOOD</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>customer request container good grade for food stuff</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M21" s="4" t="n">
@@ -3227,25 +3230,25 @@
     <row r="22" ht="13" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260900089</t>
+          <t>HASLS22260900857</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>SWIC</t>
+          <t>CMA</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2614N</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>202609211000</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="n"/>
+          <t>202609241200</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr"/>
       <c r="F22" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -3253,7 +3256,7 @@
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>TWKEL</t>
         </is>
       </c>
       <c r="H22" s="4" t="inlineStr">
@@ -3268,12 +3271,12 @@
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>SITTHINAN CO., LTD.</t>
+          <t>YUSEN LOGISTICS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
-          <t>MUNG BEAN STARCH</t>
+          <t>PRINTING FOR INDUSTRY</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
@@ -3358,68 +3361,74 @@
     <row r="23" ht="13" customHeight="1">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260900134</t>
+          <t>HASLS22260900888</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>KJT</t>
+          <t>HAB</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>202609220800</t>
-        </is>
-      </c>
-      <c r="E23" s="4" t="n"/>
+          <t>202609270600</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>THSRP</t>
+        </is>
+      </c>
       <c r="F23" s="4" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G23" s="4" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>CNSHA</t>
         </is>
       </c>
       <c r="H23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx4 </t>
         </is>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>20260912</t>
+          <t>20260916</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>THAI PLASPAC PUBLIC CO.,LTD.</t>
+          <t>FUZIN PLASTIC CO.,LTD.</t>
         </is>
       </c>
       <c r="K23" s="4" t="inlineStr">
         <is>
-          <t>PLASTIC CAP</t>
+          <t>PE RECYCLE PELLET</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>**REQUEST CLEAN AND GOOD CONTAINER</t>
+          <t>RQST CNTR 32.5 TONS // 40'HQ
+CY 16/09/2026  = 2x40'HC
+CY 18/09/2026  = 2x40'HC</t>
         </is>
       </c>
       <c r="M23" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N23" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O23" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P23" s="4" t="n">
         <v>0</v>
@@ -3487,132 +3496,132 @@
       </c>
     </row>
     <row r="24" ht="13" customHeight="1">
-      <c r="A24" s="5" t="inlineStr">
-        <is>
-          <t>HASLS22260900203</t>
-        </is>
-      </c>
-      <c r="B24" s="5" t="inlineStr">
-        <is>
-          <t>SWBT</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>2615N</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>202609211300</t>
-        </is>
-      </c>
-      <c r="E24" s="5" t="n"/>
-      <c r="F24" s="5" t="inlineStr">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260900991</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>SWMM</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>202609230900</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr"/>
+      <c r="F24" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R40Hx4 </t>
-        </is>
-      </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>20260915</t>
-        </is>
-      </c>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t>GLOBAL FROZEN FOOD (THAILAND) CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K24" s="5" t="inlineStr">
-        <is>
-          <t>FISH FROZEN</t>
-        </is>
-      </c>
-      <c r="L24" s="5" t="inlineStr">
-        <is>
-          <t>(Temp -25.0℃ / Vent Close)</t>
-        </is>
-      </c>
-      <c r="M24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="R24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="V24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="W24" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="X24" s="5">
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>RUVVO</t>
+        </is>
+      </c>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x5 </t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>20260914</t>
+        </is>
+      </c>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>RICELAND INTERNATIONAL LTD.</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>Thai Parboiled Rice 100%</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>RQST CNTR GRADE A &amp; CLEAN</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X24" s="4">
         <f>SUM(M24:U24)-V24</f>
         <v/>
       </c>
-      <c r="Y24" s="5">
+      <c r="Y24" s="4">
         <f>MAX(0,M24-MAX(0,V24))</f>
         <v/>
       </c>
-      <c r="Z24" s="5">
+      <c r="Z24" s="4">
         <f>MAX(0,N24-MAX(0,V24-SUM(M24:M24)))</f>
         <v/>
       </c>
-      <c r="AA24" s="5">
+      <c r="AA24" s="4">
         <f>MAX(0,O24-MAX(0,V24-SUM(M24:N24)))</f>
         <v/>
       </c>
-      <c r="AB24" s="5">
+      <c r="AB24" s="4">
         <f>MAX(0,P24-MAX(0,V24-SUM(M24:O24)))</f>
         <v/>
       </c>
-      <c r="AC24" s="5">
+      <c r="AC24" s="4">
         <f>MAX(0,Q24-MAX(0,V24-SUM(M24:P24)))</f>
         <v/>
       </c>
-      <c r="AD24" s="5">
+      <c r="AD24" s="4">
         <f>MAX(0,R24-MAX(0,V24-SUM(M24:Q24)))</f>
         <v/>
       </c>
-      <c r="AE24" s="5">
+      <c r="AE24" s="4">
         <f>MAX(0,S24-MAX(0,V24-SUM(M24:R24)))</f>
         <v/>
       </c>
-      <c r="AF24" s="5">
+      <c r="AF24" s="4">
         <f>MAX(0,T24-MAX(0,V24-SUM(M24:S24)))</f>
         <v/>
       </c>
-      <c r="AG24" s="5">
+      <c r="AG24" s="4">
         <f>MAX(0,U24-MAX(0,V24-SUM(M24:T24)))</f>
         <v/>
       </c>
@@ -3620,25 +3629,25 @@
     <row r="25" ht="13" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260900295</t>
+          <t>HASLS22260900992</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>KJT</t>
+          <t>SWMM</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>202609220800</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="n"/>
+          <t>202609230900</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr"/>
       <c r="F25" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -3646,12 +3655,12 @@
       </c>
       <c r="G25" s="4" t="inlineStr">
         <is>
-          <t>TWKEL</t>
+          <t>RUVVO</t>
         </is>
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">20'x5 </t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
@@ -3661,21 +3670,21 @@
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>DZQ CO.,LTD.</t>
+          <t>RICELAND INTERNATIONAL LTD.</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>FOODSTUFFS</t>
+          <t>Thai White Rice 100%</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>CONTAINER GOOD AND CLEAN</t>
+          <t>RQST CNTR GRADE A &amp; CLEAN</t>
         </is>
       </c>
       <c r="M25" s="4" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="N25" s="4" t="n">
         <v>0</v>
@@ -3751,7 +3760,7 @@
     <row r="26" ht="13" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260900311</t>
+          <t>HASLS22260901155</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
@@ -3766,7 +3775,7 @@
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>202609271400</t>
+          <t>202609270600</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -3786,58 +3795,58 @@
       </c>
       <c r="H26" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">40Hx4 </t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>20260915</t>
+          <t>20260916</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
         <is>
-          <t>SMS CORPORATION CO., LTD.</t>
+          <t>VAST OCEAN CO., LTD.</t>
         </is>
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>MODIFIED TAPIOCA STARCH</t>
+          <t>PP RECYCLE PELLET</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>FOOD GRADE CONTAINER / DO NOT RELEASE RED WALL CONTAINER</t>
+          <t>RQST CONTAINER 32.5 TONS</t>
         </is>
       </c>
       <c r="M26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="P26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V26" s="4" t="n">
         <v>2</v>
-      </c>
-      <c r="N26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V26" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="W26" s="4" t="n">
         <v>0</v>
@@ -3884,673 +3893,149 @@
       </c>
     </row>
     <row r="27" ht="13" customHeight="1">
-      <c r="A27" s="4" t="inlineStr">
-        <is>
-          <t>HASLS22260900775</t>
-        </is>
-      </c>
-      <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>SWDN</t>
-        </is>
-      </c>
-      <c r="C27" s="4" t="inlineStr">
-        <is>
-          <t>2610N</t>
-        </is>
-      </c>
-      <c r="D27" s="4" t="inlineStr">
-        <is>
-          <t>202609300900</t>
-        </is>
-      </c>
-      <c r="E27" s="4" t="n"/>
-      <c r="F27" s="4" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>KRINC</t>
-        </is>
-      </c>
-      <c r="H27" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I27" s="4" t="inlineStr">
-        <is>
-          <t>20260915</t>
-        </is>
-      </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>I-TAIL CORPORATION PUBLIC COMPANY LIMITED</t>
-        </is>
-      </c>
-      <c r="K27" s="4" t="inlineStr">
-        <is>
-          <t>PET FOOD</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M27" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W27" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X27" s="4">
-        <f>SUM(M27:U27)-V27</f>
-        <v/>
-      </c>
-      <c r="Y27" s="4">
-        <f>MAX(0,M27-MAX(0,V27))</f>
-        <v/>
-      </c>
-      <c r="Z27" s="4">
-        <f>MAX(0,N27-MAX(0,V27-SUM(M27:M27)))</f>
-        <v/>
-      </c>
-      <c r="AA27" s="4">
-        <f>MAX(0,O27-MAX(0,V27-SUM(M27:N27)))</f>
-        <v/>
-      </c>
-      <c r="AB27" s="4">
-        <f>MAX(0,P27-MAX(0,V27-SUM(M27:O27)))</f>
-        <v/>
-      </c>
-      <c r="AC27" s="4">
-        <f>MAX(0,Q27-MAX(0,V27-SUM(M27:P27)))</f>
-        <v/>
-      </c>
-      <c r="AD27" s="4">
-        <f>MAX(0,R27-MAX(0,V27-SUM(M27:Q27)))</f>
-        <v/>
-      </c>
-      <c r="AE27" s="4">
-        <f>MAX(0,S27-MAX(0,V27-SUM(M27:R27)))</f>
-        <v/>
-      </c>
-      <c r="AF27" s="4">
-        <f>MAX(0,T27-MAX(0,V27-SUM(M27:S27)))</f>
-        <v/>
-      </c>
-      <c r="AG27" s="4">
-        <f>MAX(0,U27-MAX(0,V27-SUM(M27:T27)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" ht="13" customHeight="1">
-      <c r="A28" s="4" t="inlineStr">
-        <is>
-          <t>HASLS22260900857</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
-        <is>
-          <t>CMA</t>
-        </is>
-      </c>
-      <c r="C28" s="4" t="inlineStr">
-        <is>
-          <t>2614N</t>
-        </is>
-      </c>
-      <c r="D28" s="4" t="inlineStr">
-        <is>
-          <t>202609241200</t>
-        </is>
-      </c>
-      <c r="E28" s="4" t="n"/>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>TWKEL</t>
-        </is>
-      </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I28" s="4" t="inlineStr">
-        <is>
-          <t>20260915</t>
-        </is>
-      </c>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
-          <t>YUSEN LOGISTICS (THAILAND) CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>PRINTING FOR INDUSTRY</t>
-        </is>
-      </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M28" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W28" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X28" s="4">
-        <f>SUM(M28:U28)-V28</f>
-        <v/>
-      </c>
-      <c r="Y28" s="4">
-        <f>MAX(0,M28-MAX(0,V28))</f>
-        <v/>
-      </c>
-      <c r="Z28" s="4">
-        <f>MAX(0,N28-MAX(0,V28-SUM(M28:M28)))</f>
-        <v/>
-      </c>
-      <c r="AA28" s="4">
-        <f>MAX(0,O28-MAX(0,V28-SUM(M28:N28)))</f>
-        <v/>
-      </c>
-      <c r="AB28" s="4">
-        <f>MAX(0,P28-MAX(0,V28-SUM(M28:O28)))</f>
-        <v/>
-      </c>
-      <c r="AC28" s="4">
-        <f>MAX(0,Q28-MAX(0,V28-SUM(M28:P28)))</f>
-        <v/>
-      </c>
-      <c r="AD28" s="4">
-        <f>MAX(0,R28-MAX(0,V28-SUM(M28:Q28)))</f>
-        <v/>
-      </c>
-      <c r="AE28" s="4">
-        <f>MAX(0,S28-MAX(0,V28-SUM(M28:R28)))</f>
-        <v/>
-      </c>
-      <c r="AF28" s="4">
-        <f>MAX(0,T28-MAX(0,V28-SUM(M28:S28)))</f>
-        <v/>
-      </c>
-      <c r="AG28" s="4">
-        <f>MAX(0,U28-MAX(0,V28-SUM(M28:T28)))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29" ht="13" customHeight="1">
-      <c r="A29" s="4" t="inlineStr">
-        <is>
-          <t>HASLS22260900991</t>
-        </is>
-      </c>
-      <c r="B29" s="4" t="inlineStr">
-        <is>
-          <t>SWMM</t>
-        </is>
-      </c>
-      <c r="C29" s="4" t="inlineStr">
-        <is>
-          <t>2609N</t>
-        </is>
-      </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>202609230900</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="n"/>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>RUVVO</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x5 </t>
-        </is>
-      </c>
-      <c r="I29" s="4" t="inlineStr">
-        <is>
-          <t>20260914</t>
-        </is>
-      </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>RICELAND INTERNATIONAL LTD.</t>
-        </is>
-      </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t>Thai Parboiled Rice 100%</t>
-        </is>
-      </c>
-      <c r="L29" s="4" t="inlineStr">
-        <is>
-          <t>RQST CNTR GRADE A &amp; CLEAN</t>
-        </is>
-      </c>
-      <c r="M29" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W29" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X29" s="4">
-        <f>SUM(M29:U29)-V29</f>
-        <v/>
-      </c>
-      <c r="Y29" s="4">
-        <f>MAX(0,M29-MAX(0,V29))</f>
-        <v/>
-      </c>
-      <c r="Z29" s="4">
-        <f>MAX(0,N29-MAX(0,V29-SUM(M29:M29)))</f>
-        <v/>
-      </c>
-      <c r="AA29" s="4">
-        <f>MAX(0,O29-MAX(0,V29-SUM(M29:N29)))</f>
-        <v/>
-      </c>
-      <c r="AB29" s="4">
-        <f>MAX(0,P29-MAX(0,V29-SUM(M29:O29)))</f>
-        <v/>
-      </c>
-      <c r="AC29" s="4">
-        <f>MAX(0,Q29-MAX(0,V29-SUM(M29:P29)))</f>
-        <v/>
-      </c>
-      <c r="AD29" s="4">
-        <f>MAX(0,R29-MAX(0,V29-SUM(M29:Q29)))</f>
-        <v/>
-      </c>
-      <c r="AE29" s="4">
-        <f>MAX(0,S29-MAX(0,V29-SUM(M29:R29)))</f>
-        <v/>
-      </c>
-      <c r="AF29" s="4">
-        <f>MAX(0,T29-MAX(0,V29-SUM(M29:S29)))</f>
-        <v/>
-      </c>
-      <c r="AG29" s="4">
-        <f>MAX(0,U29-MAX(0,V29-SUM(M29:T29)))</f>
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="6" t="n"/>
+      <c r="E27" s="6" t="n"/>
+      <c r="F27" s="6" t="n"/>
+      <c r="G27" s="6" t="n"/>
+      <c r="H27" s="6" t="n"/>
+      <c r="I27" s="6" t="n"/>
+      <c r="J27" s="6" t="n"/>
+      <c r="K27" s="6" t="n"/>
+      <c r="L27" s="6" t="n"/>
+      <c r="M27" s="6">
+        <f>SUM(M3:M26)</f>
+        <v/>
+      </c>
+      <c r="N27" s="6">
+        <f>SUM(N3:N26)</f>
+        <v/>
+      </c>
+      <c r="O27" s="6">
+        <f>SUM(O3:O26)</f>
+        <v/>
+      </c>
+      <c r="P27" s="6">
+        <f>SUM(P3:P26)</f>
+        <v/>
+      </c>
+      <c r="Q27" s="6">
+        <f>SUM(Q3:Q26)</f>
+        <v/>
+      </c>
+      <c r="R27" s="6">
+        <f>SUM(R3:R26)</f>
+        <v/>
+      </c>
+      <c r="S27" s="6">
+        <f>SUM(S3:S26)</f>
+        <v/>
+      </c>
+      <c r="T27" s="6">
+        <f>SUM(T3:T26)</f>
+        <v/>
+      </c>
+      <c r="U27" s="6">
+        <f>SUM(U3:U26)</f>
+        <v/>
+      </c>
+      <c r="V27" s="6">
+        <f>SUM(V3:V26)</f>
+        <v/>
+      </c>
+      <c r="W27" s="6" t="n"/>
+      <c r="X27" s="6">
+        <f>SUM(X3:X26)</f>
+        <v/>
+      </c>
+      <c r="Y27" s="6">
+        <f>SUM(Y3:Y26)</f>
+        <v/>
+      </c>
+      <c r="Z27" s="6">
+        <f>SUM(Z3:Z26)</f>
+        <v/>
+      </c>
+      <c r="AA27" s="6">
+        <f>SUM(AA3:AA26)</f>
+        <v/>
+      </c>
+      <c r="AB27" s="6">
+        <f>SUM(AB3:AB26)</f>
+        <v/>
+      </c>
+      <c r="AC27" s="6">
+        <f>SUM(AC3:AC26)</f>
+        <v/>
+      </c>
+      <c r="AD27" s="6">
+        <f>SUM(AD3:AD26)</f>
+        <v/>
+      </c>
+      <c r="AE27" s="6">
+        <f>SUM(AE3:AE26)</f>
+        <v/>
+      </c>
+      <c r="AF27" s="6">
+        <f>SUM(AF3:AF26)</f>
+        <v/>
+      </c>
+      <c r="AG27" s="6">
+        <f>SUM(AG3:AG26)</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="13" customHeight="1">
-      <c r="A30" s="4" t="inlineStr">
-        <is>
-          <t>HASLS22260900992</t>
-        </is>
-      </c>
-      <c r="B30" s="4" t="inlineStr">
-        <is>
-          <t>SWMM</t>
-        </is>
-      </c>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>2609N</t>
-        </is>
-      </c>
-      <c r="D30" s="4" t="inlineStr">
-        <is>
-          <t>202609230900</t>
-        </is>
-      </c>
-      <c r="E30" s="4" t="n"/>
-      <c r="F30" s="4" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>RUVVO</t>
-        </is>
-      </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x5 </t>
-        </is>
-      </c>
-      <c r="I30" s="4" t="inlineStr">
-        <is>
-          <t>20260914</t>
-        </is>
-      </c>
-      <c r="J30" s="4" t="inlineStr">
-        <is>
-          <t>RICELAND INTERNATIONAL LTD.</t>
-        </is>
-      </c>
-      <c r="K30" s="4" t="inlineStr">
-        <is>
-          <t>Thai White Rice 100%</t>
-        </is>
-      </c>
-      <c r="L30" s="4" t="inlineStr">
-        <is>
-          <t>RQST CNTR GRADE A &amp; CLEAN</t>
-        </is>
-      </c>
-      <c r="M30" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="V30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W30" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="X30" s="4">
-        <f>SUM(M30:U30)-V30</f>
-        <v/>
-      </c>
-      <c r="Y30" s="4">
-        <f>MAX(0,M30-MAX(0,V30))</f>
-        <v/>
-      </c>
-      <c r="Z30" s="4">
-        <f>MAX(0,N30-MAX(0,V30-SUM(M30:M30)))</f>
-        <v/>
-      </c>
-      <c r="AA30" s="4">
-        <f>MAX(0,O30-MAX(0,V30-SUM(M30:N30)))</f>
-        <v/>
-      </c>
-      <c r="AB30" s="4">
-        <f>MAX(0,P30-MAX(0,V30-SUM(M30:O30)))</f>
-        <v/>
-      </c>
-      <c r="AC30" s="4">
-        <f>MAX(0,Q30-MAX(0,V30-SUM(M30:P30)))</f>
-        <v/>
-      </c>
-      <c r="AD30" s="4">
-        <f>MAX(0,R30-MAX(0,V30-SUM(M30:Q30)))</f>
-        <v/>
-      </c>
-      <c r="AE30" s="4">
-        <f>MAX(0,S30-MAX(0,V30-SUM(M30:R30)))</f>
-        <v/>
-      </c>
-      <c r="AF30" s="4">
-        <f>MAX(0,T30-MAX(0,V30-SUM(M30:S30)))</f>
-        <v/>
-      </c>
-      <c r="AG30" s="4">
-        <f>MAX(0,U30-MAX(0,V30-SUM(M30:T30)))</f>
-        <v/>
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B30" s="7" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C30" s="7" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
       </c>
     </row>
     <row r="31" ht="13" customHeight="1">
-      <c r="A31" s="6" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B31" s="6" t="n"/>
-      <c r="C31" s="6" t="n"/>
-      <c r="D31" s="6" t="n"/>
-      <c r="E31" s="6" t="n"/>
-      <c r="F31" s="6" t="n"/>
-      <c r="G31" s="6" t="n"/>
-      <c r="H31" s="6" t="n"/>
-      <c r="I31" s="6" t="n"/>
-      <c r="J31" s="6" t="n"/>
-      <c r="K31" s="6" t="n"/>
-      <c r="L31" s="6" t="n"/>
-      <c r="M31" s="6">
-        <f>SUM(M3:M30)</f>
-        <v/>
-      </c>
-      <c r="N31" s="6">
-        <f>SUM(N3:N30)</f>
-        <v/>
-      </c>
-      <c r="O31" s="6">
-        <f>SUM(O3:O30)</f>
-        <v/>
-      </c>
-      <c r="P31" s="6">
-        <f>SUM(P3:P30)</f>
-        <v/>
-      </c>
-      <c r="Q31" s="6">
-        <f>SUM(Q3:Q30)</f>
-        <v/>
-      </c>
-      <c r="R31" s="6">
-        <f>SUM(R3:R30)</f>
-        <v/>
-      </c>
-      <c r="S31" s="6">
-        <f>SUM(S3:S30)</f>
-        <v/>
-      </c>
-      <c r="T31" s="6">
-        <f>SUM(T3:T30)</f>
-        <v/>
-      </c>
-      <c r="U31" s="6">
-        <f>SUM(U3:U30)</f>
-        <v/>
-      </c>
-      <c r="V31" s="6">
-        <f>SUM(V3:V30)</f>
-        <v/>
-      </c>
-      <c r="W31" s="6" t="n"/>
-      <c r="X31" s="6">
-        <f>SUM(X3:X30)</f>
-        <v/>
-      </c>
-      <c r="Y31" s="6">
-        <f>SUM(Y3:Y30)</f>
-        <v/>
-      </c>
-      <c r="Z31" s="6">
-        <f>SUM(Z3:Z30)</f>
-        <v/>
-      </c>
-      <c r="AA31" s="6">
-        <f>SUM(AA3:AA30)</f>
-        <v/>
-      </c>
-      <c r="AB31" s="6">
-        <f>SUM(AB3:AB30)</f>
-        <v/>
-      </c>
-      <c r="AC31" s="6">
-        <f>SUM(AC3:AC30)</f>
-        <v/>
-      </c>
-      <c r="AD31" s="6">
-        <f>SUM(AD3:AD30)</f>
-        <v/>
-      </c>
-      <c r="AE31" s="6">
-        <f>SUM(AE3:AE30)</f>
-        <v/>
-      </c>
-      <c r="AF31" s="6">
-        <f>SUM(AF3:AF30)</f>
-        <v/>
-      </c>
-      <c r="AG31" s="6">
-        <f>SUM(AG3:AG30)</f>
-        <v/>
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>B.C. DEPOT CO.,LTD. ( Bang-Na KM.18)</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="C31" s="4" t="n">
+        <v>85</v>
       </c>
     </row>
-    <row r="34" ht="13" customHeight="1">
-      <c r="A34" s="7" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C34" s="7" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="13" customHeight="1">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t>B.C. DEPOT CO.,LTD. ( Bang-Na KM.18)</t>
-        </is>
-      </c>
-      <c r="B35" s="4" t="n">
-        <v>28</v>
-      </c>
-      <c r="C35" s="4" t="n">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="36" ht="13" customHeight="1">
-      <c r="A36" s="6" t="inlineStr">
+    <row r="32" ht="13" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B36" s="6" t="n">
-        <v>28</v>
-      </c>
-      <c r="C36" s="6" t="n">
-        <v>86</v>
+      <c r="B32" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="C32" s="6" t="n">
+        <v>85</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:AG30"/>
+  <autoFilter ref="A2:AG26"/>
   <mergeCells count="1">
     <mergeCell ref="A1:AG1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Rename Remaining columns to plain type names in per-pickup files
"GP22 Remaining" etc. -> "GP22" (and so on for all 9 type columns)
in the per-depot files, since the raw booked-qty columns were
already removed and these are now the only per-type figures shown.
Column widths recompute automatically from the shorter headers
(autofit rule unchanged: tight to content, ORG CUST/COMMODITY/
TRAFFIC ORDER stay fixed-wide).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - B.C. DEPOT CO.,LTD. ( Bang-Na KM.18).xlsx
+++ b/output/bkg pending - B.C. DEPOT CO.,LTD. ( Bang-Na KM.18).xlsx
@@ -507,15 +507,15 @@
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
     <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="16" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="16" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
-    <col width="16" customWidth="1" min="20" max="20"/>
-    <col width="16" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="13" customHeight="1">
@@ -608,47 +608,47 @@
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>GP22 Remaining</t>
+          <t>GP22</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t>GP42 Remaining</t>
+          <t>GP42</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t>GP45 Remaining</t>
+          <t>GP45</t>
         </is>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>RE22 Remaining</t>
+          <t>RE22</t>
         </is>
       </c>
       <c r="Q2" s="3" t="inlineStr">
         <is>
-          <t>RE45 Remaining</t>
+          <t>RE45</t>
         </is>
       </c>
       <c r="R2" s="3" t="inlineStr">
         <is>
-          <t>UT22 Remaining</t>
+          <t>UT22</t>
         </is>
       </c>
       <c r="S2" s="3" t="inlineStr">
         <is>
-          <t>UT42 Remaining</t>
+          <t>UT42</t>
         </is>
       </c>
       <c r="T2" s="3" t="inlineStr">
         <is>
-          <t>PC22 Remaining</t>
+          <t>PC22</t>
         </is>
       </c>
       <c r="U2" s="3" t="inlineStr">
         <is>
-          <t>PC42 Remaining</t>
+          <t>PC42</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update dashboard and reports with 9-17-PD booking data
Regenerated from "9-17-PD.xls" (2839 rows): 125 BK No outstanding,
294 containers. HASLS22260900416 is still flagged for missing
Pickup Name — now unresolved for 6 consecutive days of data.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - B.C. DEPOT CO.,LTD. ( Bang-Na KM.18).xlsx
+++ b/output/bkg pending - B.C. DEPOT CO.,LTD. ( Bang-Na KM.18).xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$2:$U$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$2:$U$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U32"/>
+  <dimension ref="A1:U40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -502,7 +502,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
@@ -655,25 +655,25 @@
     <row r="3" ht="13" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260800253</t>
+          <t>HASLS22260800546</t>
         </is>
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>SWBT</t>
+          <t>SWMM</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>2615N</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D3" s="4" t="inlineStr">
         <is>
-          <t>202609210900</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="n"/>
+          <t>202609221300</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr"/>
       <c r="F3" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -686,37 +686,37 @@
       </c>
       <c r="H3" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">40Hx2 </t>
         </is>
       </c>
       <c r="I3" s="4" t="inlineStr">
         <is>
-          <t>20260914</t>
+          <t>20260917</t>
         </is>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
-          <t>UENO FINE CHEMICALS INDUSTRY (THAILAND) LTD.</t>
+          <t>PANASONIC MANUFACTURING AYUTHAYA CO., LTD.</t>
         </is>
       </c>
       <c r="K3" s="4" t="inlineStr">
         <is>
-          <t>MALTITOL SYRUP</t>
+          <t>AMINO FORMALDEHYDE COMPOUNDS (UREA)</t>
         </is>
       </c>
       <c r="L3" s="4" t="inlineStr">
         <is>
-          <t>Req food grade container due to commodity is food stuff.</t>
+          <t>GOOD GRADE CONTAINER with STRONG FLOOR</t>
         </is>
       </c>
       <c r="M3" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N3" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O3" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P3" s="4" t="n">
         <v>0</v>
@@ -740,25 +740,25 @@
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801252</t>
+          <t>HASLS22260800749</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>KJT</t>
+          <t>SWMM</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>202609222100</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="n"/>
+          <t>202609221300</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr"/>
       <c r="F4" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -766,36 +766,36 @@
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>JPMYJ</t>
         </is>
       </c>
       <c r="H4" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x4 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>20260910</t>
+          <t>20260917</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>CHEVRON (THAILAND) LIMITED</t>
+          <t>GENERAL FOOD PRODUCTS CO., LTD.</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>LUBE OIL</t>
+          <t>FLOURS</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Req. Container condition  GRADE B+ CNTR / CLEAN CNTR WITH GOOD CONDITION / NO SMELL/NODAMAGES / STRONG &amp; SMOOTH FLOOR / NO NAILS / LOAD UNDERDECK</t>
+          <t>Container Grade A</t>
         </is>
       </c>
       <c r="M4" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>0</v>
@@ -825,25 +825,25 @@
     <row r="5" ht="13" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801423</t>
+          <t>HASLS22260800754</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>KMGY</t>
+          <t>KUS</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2615N</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>202609271700</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="n"/>
+          <t>202609231100</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr"/>
       <c r="F5" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -851,42 +851,42 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>CNXMN</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x2 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>20260915</t>
+          <t>20260917</t>
         </is>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
-          <t>TAKO FOODS INDUSTRY CO., LTD.</t>
+          <t>SIAM FUKOKU CO.,LTD.</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
         <is>
-          <t>COCONUT WATER</t>
+          <t>BLADE RUBBER</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>RQS CLEAN &amp; GOOD CONTAINER CONDITION.</t>
         </is>
       </c>
       <c r="M5" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N5" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O5" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P5" s="4" t="n">
         <v>0</v>
@@ -910,72 +910,68 @@
     <row r="6" ht="13" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801587</t>
+          <t>HASLS22260801169</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>NSSJ</t>
+          <t>SWMM</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>2607S</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>202609220800</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>THLKR</t>
-        </is>
-      </c>
+          <t>202609221300</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr"/>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>THLCH</t>
+          <t>THBKK</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
         <is>
-          <t>IDJKT</t>
+          <t>KRPUS</t>
         </is>
       </c>
       <c r="H6" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx4 </t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>20260912</t>
+          <t>20260917</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
         <is>
-          <t>MEDIFOODS (THAILAND) CO., LTD.</t>
+          <t>THAI ASAHI CO., LTD.</t>
         </is>
       </c>
       <c r="K6" s="4" t="inlineStr">
         <is>
-          <t>ORGANIC JASMINE RICE FLOUR 120MESH</t>
+          <t xml:space="preserve">POTATO STARCH </t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>GOOD &amp; CLEAN CONTAINER</t>
+          <t>Grade A and food grade container</t>
         </is>
       </c>
       <c r="M6" s="4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N6" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O6" s="4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="P6" s="4" t="n">
         <v>0</v>
@@ -999,25 +995,25 @@
     <row r="7" ht="13" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801914</t>
+          <t>HASLS22260801423</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>SWMM</t>
+          <t>KMGY</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>202609230900</t>
-        </is>
-      </c>
-      <c r="E7" s="4" t="n"/>
+          <t>202609290000</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr"/>
       <c r="F7" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -1025,12 +1021,12 @@
       </c>
       <c r="G7" s="4" t="inlineStr">
         <is>
-          <t>KRPTK</t>
+          <t>CNXMN</t>
         </is>
       </c>
       <c r="H7" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x33 </t>
+          <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
       <c r="I7" s="4" t="inlineStr">
@@ -1040,22 +1036,21 @@
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
-          <t>DP WORLD LOGISTICS SOLUTIONS (THAILAND) COMPANY LIMITED</t>
+          <t>TAKO FOODS INDUSTRY CO., LTD.</t>
         </is>
       </c>
       <c r="K7" s="4" t="inlineStr">
         <is>
-          <t>SOYBEAN OIL</t>
+          <t>COCONUT WATER</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>** APPROVAL MR.KIM GEON WOOK DD.25/08/2026  ** *FLEXIBAG ONDECK*
-Servey: 15/09/2026, Pickup : 16/09/2026</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M7" s="4" t="n">
-        <v>33</v>
+        <v>2</v>
       </c>
       <c r="N7" s="4" t="n">
         <v>0</v>
@@ -1085,12 +1080,12 @@
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260801939</t>
+          <t>HASLS22260801643</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>SWSP</t>
+          <t>SWMM</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1100,10 +1095,10 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>202610022300</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="n"/>
+          <t>202609221300</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr"/>
       <c r="F8" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -1116,31 +1111,31 @@
       </c>
       <c r="H8" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x7 </t>
+          <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
         <is>
-          <t>20260907</t>
+          <t>20260917</t>
         </is>
       </c>
       <c r="J8" s="4" t="inlineStr">
         <is>
-          <t>THAI GYPSUM PRODUCTS PCL.</t>
+          <t>UENO FINE CHEMICALS INDUSTRY (THAILAND) LTD.</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
         <is>
-          <t>GYPSUM PLASTER - 25202090</t>
+          <t>MALTITOL SYRUP</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>Req food grade container due to commodity is food stuff.</t>
         </is>
       </c>
       <c r="M8" s="4" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="N8" s="4" t="n">
         <v>0</v>
@@ -1170,25 +1165,25 @@
     <row r="9" ht="13" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260802080</t>
+          <t>HASLS22260801914</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>SWIC</t>
+          <t>SWMM</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>202609211200</t>
-        </is>
-      </c>
-      <c r="E9" s="4" t="n"/>
+          <t>202609221300</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr"/>
       <c r="F9" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -1196,36 +1191,37 @@
       </c>
       <c r="G9" s="4" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>KRPTK</t>
         </is>
       </c>
       <c r="H9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x14 </t>
+          <t xml:space="preserve">20'x33 </t>
         </is>
       </c>
       <c r="I9" s="4" t="inlineStr">
         <is>
-          <t>20260916</t>
+          <t>20260917</t>
         </is>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>THAI FERMENTATION INDUSTRY CO., LTD.</t>
+          <t>DP WORLD LOGISTICS SOLUTIONS (THAILAND) COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
         <is>
-          <t>MSG</t>
+          <t>SOYBEAN OIL</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>REQ food grate ctn</t>
+          <t>** APPROVAL MR.KIM GEON WOOK DD.25/08/2026  ** *FLEXIBAG ONDECK*
+Servey: 17/09/2026, Pickup : 18/09/2026</t>
         </is>
       </c>
       <c r="M9" s="4" t="n">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="N9" s="4" t="n">
         <v>0</v>
@@ -1255,633 +1251,629 @@
     <row r="10" ht="13" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260802148</t>
+          <t>HASLS22260801939</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>KJT</t>
+          <t>SWSP</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>202610040200</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr"/>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>THBKK</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x7 </t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>20260907</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>THAI GYPSUM PRODUCTS PCL.</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>GYPSUM PLASTER - 25202090</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U10" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="13" customHeight="1">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260802081</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>SWIC</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
           <t>2610N</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>202609222100</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="n"/>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>202609211300</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr"/>
+      <c r="F11" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G10" s="4" t="inlineStr">
-        <is>
-          <t>HKHKG</t>
-        </is>
-      </c>
-      <c r="H10" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I10" s="4" t="inlineStr">
-        <is>
-          <t>20260916</t>
-        </is>
-      </c>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>SINGHA WORLDWIDE INTERNATIONAL CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>SODA WATER</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>Under desk cargo and food grade container</t>
-        </is>
-      </c>
-      <c r="M10" s="4" t="n">
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x14 </t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
+        <is>
+          <t>20260917</t>
+        </is>
+      </c>
+      <c r="J11" s="4" t="inlineStr">
+        <is>
+          <t>THAI FERMENTATION INDUSTRY CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>MSG</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>REQ food grate ctn</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="N10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T10" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U10" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" ht="13" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>HASLS22260802265</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>CMA</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>2614N</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>202609241200</t>
-        </is>
-      </c>
-      <c r="E11" s="5" t="n"/>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="N11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="13" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260802255</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>SWIC</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>202609211300</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr"/>
+      <c r="F12" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
-        <is>
-          <t>HKHKG</t>
-        </is>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R40Hx1 </t>
-        </is>
-      </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>20260914</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>KIBUN (THAILAND) CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>FROZEN IMITATION CRAB MEAT</t>
-        </is>
-      </c>
-      <c r="L11" s="5" t="inlineStr">
-        <is>
-          <t>(Temp -20.0 / Vent Close)  **REQ GOOD, CLEAN, NO LEAK AND GRADE A CONTAINER</t>
-        </is>
-      </c>
-      <c r="M11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="R11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U11" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" ht="13" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
-        <is>
-          <t>HASLS22260802566</t>
-        </is>
-      </c>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>SWAT</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>2611N</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>202610251024</t>
-        </is>
-      </c>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>KRPUS</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R40Hx1 </t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>20260916</t>
-        </is>
-      </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>N&amp;N FOODS CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>FROZEN FOOD</t>
-        </is>
-      </c>
-      <c r="L12" s="5" t="inlineStr">
-        <is>
-          <t>(Temp -20.0℃ / Vent Close) Request good and clean container</t>
-        </is>
-      </c>
-      <c r="M12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="R12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U12" s="5" t="n">
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx3 </t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>20260917</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>EXCEL ENTECH CO.,LTD.</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>PARTS OF MACHINERY</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U12" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="13" ht="13" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
         <is>
+          <t>HASLS22260802265</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>CMA</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>2614N</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>202609240200</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr"/>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>THBKK</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="inlineStr">
+        <is>
+          <t>HKHKG</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R40Hx1 </t>
+        </is>
+      </c>
+      <c r="I13" s="5" t="inlineStr">
+        <is>
+          <t>20260914</t>
+        </is>
+      </c>
+      <c r="J13" s="5" t="inlineStr">
+        <is>
+          <t>KIBUN (THAILAND) CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K13" s="5" t="inlineStr">
+        <is>
+          <t>FROZEN IMITATION CRAB MEAT</t>
+        </is>
+      </c>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>(Temp -20.0 / Vent Close)  **REQ GOOD, CLEAN, NO LEAK AND GRADE A CONTAINER</t>
+        </is>
+      </c>
+      <c r="M13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="R13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U13" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="13" customHeight="1">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260802436</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>KUS</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>2615N</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>202609231100</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr"/>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>THBKK</t>
+        </is>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
+          <t>JPSEN</t>
+        </is>
+      </c>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr">
+        <is>
+          <t>20260917</t>
+        </is>
+      </c>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>TANIO THAI CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>RED BEAN PASTE</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>RQST CNTR FOOD GRADE</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="13" customHeight="1">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>HASLS22260802566</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>SWAT</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>2611N</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>202610251024</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr"/>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>THBKK</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>KRPUS</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R40Hx1 </t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>20260916</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>N&amp;N FOODS CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>FROZEN FOOD</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>(Temp -20.0℃ / Vent Close) Request good and clean container</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="R15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U15" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="13" customHeight="1">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
           <t>HASLS22260802575</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B16" s="5" t="inlineStr">
         <is>
           <t>SWIC</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C16" s="5" t="inlineStr">
         <is>
           <t>2610N</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>202609211200</t>
-        </is>
-      </c>
-      <c r="E13" s="5" t="n"/>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>202609211300</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr"/>
+      <c r="F16" s="5" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G16" s="5" t="inlineStr">
         <is>
           <t>VNSGN</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H16" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">R40Hx6 </t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="I16" s="5" t="inlineStr">
         <is>
           <t>20260914</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="J16" s="5" t="inlineStr">
         <is>
           <t>GOLDEN PRIZE CANNING CO., LTD.</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="K16" s="5" t="inlineStr">
         <is>
           <t>FROZEN TUNA</t>
         </is>
       </c>
-      <c r="L13" s="5" t="inlineStr">
+      <c r="L16" s="5" t="inlineStr">
         <is>
           <t>(Temp -25.0℃ / Vent Close)
 REQUEST GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
-      <c r="M13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="R13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U13" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" ht="13" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>HASLS22260900037</t>
-        </is>
-      </c>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>KUS</t>
-        </is>
-      </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>2615N</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>202609222100</t>
-        </is>
-      </c>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="5" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G14" s="5" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H14" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R40Hx2 </t>
-        </is>
-      </c>
-      <c r="I14" s="5" t="inlineStr">
-        <is>
-          <t>20260916</t>
-        </is>
-      </c>
-      <c r="J14" s="5" t="inlineStr">
-        <is>
-          <t>INVE (THAILAND) LTD</t>
-        </is>
-      </c>
-      <c r="K14" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ANIMAL FEED </t>
-        </is>
-      </c>
-      <c r="L14" s="5" t="inlineStr">
-        <is>
-          <t>(Temp +2.0℃ / Vent Close) REQUEST GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="5" t="n">
+      <c r="M16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="R14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U14" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" ht="13" customHeight="1">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>HASLS22260900089</t>
-        </is>
-      </c>
-      <c r="B15" s="4" t="inlineStr">
-        <is>
-          <t>SWIC</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
-        <is>
-          <t>2610N</t>
-        </is>
-      </c>
-      <c r="D15" s="4" t="inlineStr">
-        <is>
-          <t>202609211200</t>
-        </is>
-      </c>
-      <c r="E15" s="4" t="n"/>
-      <c r="F15" s="4" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H15" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I15" s="4" t="inlineStr">
-        <is>
-          <t>20260915</t>
-        </is>
-      </c>
-      <c r="J15" s="4" t="inlineStr">
-        <is>
-          <t>SITTHINAN CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K15" s="4" t="inlineStr">
-        <is>
-          <t>MUNG BEAN STARCH</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T15" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U15" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" ht="13" customHeight="1">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>HASLS22260900295</t>
-        </is>
-      </c>
-      <c r="B16" s="4" t="inlineStr">
-        <is>
-          <t>KJT</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
-        <is>
-          <t>2610N</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="inlineStr">
-        <is>
-          <t>202609222100</t>
-        </is>
-      </c>
-      <c r="E16" s="4" t="n"/>
-      <c r="F16" s="4" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>TWKEL</t>
-        </is>
-      </c>
-      <c r="H16" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I16" s="4" t="inlineStr">
-        <is>
-          <t>20260914</t>
-        </is>
-      </c>
-      <c r="J16" s="4" t="inlineStr">
-        <is>
-          <t>DZQ CO.,LTD.</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>FOODSTUFFS</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>CONTAINER GOOD AND CLEAN</t>
-        </is>
-      </c>
-      <c r="M16" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="N16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U16" s="4" t="n">
+      <c r="R16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="T16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="U16" s="5" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="17" ht="13" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260900311</t>
+          <t>HASLS22260900121</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>HAB</t>
+          <t>KMGY</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>202609270600</t>
-        </is>
-      </c>
-      <c r="E17" s="4" t="inlineStr">
-        <is>
-          <t>THSRP</t>
-        </is>
-      </c>
+          <t>202609290000</t>
+        </is>
+      </c>
+      <c r="E17" s="4" t="inlineStr"/>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>THLCH</t>
+          <t>THBKK</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>CNXMN</t>
         </is>
       </c>
       <c r="H17" s="4" t="inlineStr">
@@ -1891,22 +1883,22 @@
       </c>
       <c r="I17" s="4" t="inlineStr">
         <is>
-          <t>20260915</t>
+          <t>20260917</t>
         </is>
       </c>
       <c r="J17" s="4" t="inlineStr">
         <is>
-          <t>SMS CORPORATION CO., LTD.</t>
+          <t>NITTO FUJI INTERNATIONAL (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K17" s="4" t="inlineStr">
         <is>
-          <t>MODIFIED TAPIOCA STARCH</t>
+          <t>MIX FLOUR</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>FOOD GRADE CONTAINER / DO NOT RELEASE RED WALL CONTAINER</t>
+          <t>REQUEST GOOD, CLEAN AND NO SMELL CONTAINER / REQUEST FOOD GRADE CONTAINER</t>
         </is>
       </c>
       <c r="M17" s="4" t="n">
@@ -1940,7 +1932,7 @@
     <row r="18" ht="13" customHeight="1">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260900552</t>
+          <t>HASLS22260900295</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -1955,10 +1947,10 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>202609222100</t>
-        </is>
-      </c>
-      <c r="E18" s="4" t="n"/>
+          <t>202609221900</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr"/>
       <c r="F18" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -1966,42 +1958,42 @@
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>CNSHK</t>
+          <t>TWKEL</t>
         </is>
       </c>
       <c r="H18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx2 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>20260916</t>
+          <t>20260914</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
         <is>
-          <t>NMB-MINEBEA THAI LTD.</t>
+          <t>DZQ CO.,LTD.</t>
         </is>
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>BALL BEARING</t>
+          <t>FOODSTUFFS</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>REQUEST CLEAN CONTAINER</t>
+          <t>CONTAINER GOOD AND CLEAN</t>
         </is>
       </c>
       <c r="M18" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N18" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O18" s="4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P18" s="4" t="n">
         <v>0</v>
@@ -2023,184 +2015,184 @@
       </c>
     </row>
     <row r="19" ht="13" customHeight="1">
-      <c r="A19" s="5" t="inlineStr">
-        <is>
-          <t>HASLS22260900747</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>SWBT</t>
-        </is>
-      </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>2615N</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>202609210900</t>
-        </is>
-      </c>
-      <c r="E19" s="5" t="n"/>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260900335</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>KMGY</t>
+        </is>
+      </c>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>202609290000</t>
+        </is>
+      </c>
+      <c r="E19" s="4" t="inlineStr"/>
+      <c r="F19" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H19" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R40Hx1 </t>
-        </is>
-      </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>20260916</t>
-        </is>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>MEGA LIFESCIENCES PUBLIC CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K19" s="5" t="inlineStr">
-        <is>
-          <t>PHARMACEUTICAL PRODUCTS</t>
-        </is>
-      </c>
-      <c r="L19" s="5" t="inlineStr">
-        <is>
-          <t>Temp  +22.0℃ / Vent Close)</t>
-        </is>
-      </c>
-      <c r="M19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="5" t="n">
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>HKHKG</t>
+        </is>
+      </c>
+      <c r="H19" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x5 </t>
+        </is>
+      </c>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>20260917</t>
+        </is>
+      </c>
+      <c r="J19" s="4" t="inlineStr">
+        <is>
+          <t>PERFECT LEATHER CO.,LTD.</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>WET BLUE CATTLE HIDES</t>
+        </is>
+      </c>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M19" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T19" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U19" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="13" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260900775</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>SWDN</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>2610N</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>202609300900</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr"/>
+      <c r="F20" s="4" t="inlineStr">
+        <is>
+          <t>THBKK</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>KRINC</t>
+        </is>
+      </c>
+      <c r="H20" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I20" s="4" t="inlineStr">
+        <is>
+          <t>20260915</t>
+        </is>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>I-TAIL CORPORATION PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>PET FOOD</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M20" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="R19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U19" s="5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" ht="13" customHeight="1">
-      <c r="A20" s="5" t="inlineStr">
-        <is>
-          <t>HASLS22260900748</t>
-        </is>
-      </c>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>SWBT</t>
-        </is>
-      </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>2615N</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>202609210900</t>
-        </is>
-      </c>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="5" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G20" s="5" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H20" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R40Hx1 </t>
-        </is>
-      </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>20260916</t>
-        </is>
-      </c>
-      <c r="J20" s="5" t="inlineStr">
-        <is>
-          <t>MEGA LIFESCIENCES PUBLIC CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K20" s="5" t="inlineStr">
-        <is>
-          <t>PHARMACEUTICAL PRODUCTS</t>
-        </is>
-      </c>
-      <c r="L20" s="5" t="inlineStr">
-        <is>
-          <t>(Temp +22.0℃ / Vent Close)</t>
-        </is>
-      </c>
-      <c r="M20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q20" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="R20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="T20" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U20" s="5" t="n">
+      <c r="N20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U20" s="4" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21" ht="13" customHeight="1">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260900775</t>
+          <t>HASLS22260900832</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>SWDN</t>
+          <t>SWIC</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -2210,10 +2202,10 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>202609300900</t>
-        </is>
-      </c>
-      <c r="E21" s="4" t="n"/>
+          <t>202609211300</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr"/>
       <c r="F21" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -2221,42 +2213,42 @@
       </c>
       <c r="G21" s="4" t="inlineStr">
         <is>
-          <t>KRINC</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I21" s="4" t="inlineStr">
         <is>
-          <t>20260915</t>
+          <t>20260917</t>
         </is>
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>I-TAIL CORPORATION PUBLIC COMPANY LIMITED</t>
+          <t>TETRA PAK (THAILAND) LIMITED</t>
         </is>
       </c>
       <c r="K21" s="4" t="inlineStr">
         <is>
-          <t>PET FOOD</t>
+          <t>USED PLASTIC PALLET</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>REQUEST CONTAINER GOODS &amp; CLEAN</t>
         </is>
       </c>
       <c r="M21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="4" t="n">
         <v>1</v>
-      </c>
-      <c r="N21" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="4" t="n">
-        <v>0</v>
       </c>
       <c r="P21" s="4" t="n">
         <v>0</v>
@@ -2295,10 +2287,10 @@
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>202609241200</t>
-        </is>
-      </c>
-      <c r="E22" s="4" t="n"/>
+          <t>202609240200</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr"/>
       <c r="F22" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -2456,25 +2448,25 @@
     <row r="24" ht="13" customHeight="1">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260900991</t>
+          <t>HASLS22260900893</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>SWMM</t>
+          <t>CMA</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2614N</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>202609230900</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="n"/>
+          <t>202609240200</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr"/>
       <c r="F24" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -2482,36 +2474,36 @@
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>RUVVO</t>
+          <t>TWKEL</t>
         </is>
       </c>
       <c r="H24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x5 </t>
+          <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>20260914</t>
+          <t>20260917</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>RICELAND INTERNATIONAL LTD.</t>
+          <t>SMS CORPORATION CO., LTD.</t>
         </is>
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>Thai Parboiled Rice 100%</t>
+          <t xml:space="preserve">MODIFIED TAPIOCA STARCH </t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>RQST CNTR GRADE A &amp; CLEAN</t>
+          <t>NEED VERY CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M24" s="4" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="N24" s="4" t="n">
         <v>0</v>
@@ -2541,25 +2533,25 @@
     <row r="25" ht="13" customHeight="1">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260900992</t>
+          <t>HASLS22260900894</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>SWMM</t>
+          <t>KUS</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2615N</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>202609230900</t>
-        </is>
-      </c>
-      <c r="E25" s="4" t="n"/>
+          <t>202609231100</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr"/>
       <c r="F25" s="4" t="inlineStr">
         <is>
           <t>THBKK</t>
@@ -2572,37 +2564,37 @@
       </c>
       <c r="H25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x5 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I25" s="4" t="inlineStr">
         <is>
-          <t>20260914</t>
+          <t>20260917</t>
         </is>
       </c>
       <c r="J25" s="4" t="inlineStr">
         <is>
-          <t>RICELAND INTERNATIONAL LTD.</t>
+          <t>PENTA IMPEX CO.,LTD.</t>
         </is>
       </c>
       <c r="K25" s="4" t="inlineStr">
         <is>
-          <t>Thai White Rice 100%</t>
+          <t>GENERAL FOODSTUFFS (SAUCE)</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>RQST CNTR GRADE A &amp; CLEAN</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M25" s="4" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="N25" s="4" t="n">
         <v>0</v>
       </c>
       <c r="O25" s="4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P25" s="4" t="n">
         <v>0</v>
@@ -2626,191 +2618,879 @@
     <row r="26" ht="13" customHeight="1">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>HASLS22260901155</t>
+          <t>HASLS22260900923</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
+          <t>CMA</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>2614N</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>202609240200</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr"/>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>THBKK</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>TWKEL</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>20260917</t>
+        </is>
+      </c>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>YUTO-COSMO (THAILAND) CO.,LTD</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U26" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" ht="13" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260900991</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>SWMM</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>202609221300</t>
+        </is>
+      </c>
+      <c r="E27" s="4" t="inlineStr"/>
+      <c r="F27" s="4" t="inlineStr">
+        <is>
+          <t>THBKK</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>RUVVO</t>
+        </is>
+      </c>
+      <c r="H27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x5 </t>
+        </is>
+      </c>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>20260914</t>
+        </is>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>RICELAND INTERNATIONAL LTD.</t>
+        </is>
+      </c>
+      <c r="K27" s="4" t="inlineStr">
+        <is>
+          <t>Thai Parboiled Rice 100%</t>
+        </is>
+      </c>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>RQST CNTR GRADE A &amp; CLEAN</t>
+        </is>
+      </c>
+      <c r="M27" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U27" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" ht="13" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260900992</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>SWMM</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>202609221300</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr"/>
+      <c r="F28" s="4" t="inlineStr">
+        <is>
+          <t>THBKK</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>RUVVO</t>
+        </is>
+      </c>
+      <c r="H28" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x5 </t>
+        </is>
+      </c>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>20260914</t>
+        </is>
+      </c>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>RICELAND INTERNATIONAL LTD.</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>Thai White Rice 100%</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>RQST CNTR GRADE A &amp; CLEAN</t>
+        </is>
+      </c>
+      <c r="M28" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U28" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" ht="13" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260901067</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
           <t>HAB</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>2611N</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D29" s="4" t="inlineStr">
         <is>
           <t>202609270600</t>
         </is>
       </c>
-      <c r="E26" s="4" t="inlineStr">
+      <c r="E29" s="4" t="inlineStr">
         <is>
           <t>THSRP</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="F29" s="4" t="inlineStr">
         <is>
           <t>THLCH</t>
         </is>
       </c>
-      <c r="G26" s="4" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
         <is>
           <t>CNSHA</t>
         </is>
       </c>
-      <c r="H26" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40Hx4 </t>
-        </is>
-      </c>
-      <c r="I26" s="4" t="inlineStr">
-        <is>
-          <t>20260916</t>
-        </is>
-      </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>VAST OCEAN CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>PP RECYCLE PELLET</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>RQST CONTAINER 32.5 TONS</t>
-        </is>
-      </c>
-      <c r="M26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="P26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="R26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T26" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="U26" s="4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" ht="13" customHeight="1">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="n"/>
-      <c r="C27" s="6" t="n"/>
-      <c r="D27" s="6" t="n"/>
-      <c r="E27" s="6" t="n"/>
-      <c r="F27" s="6" t="n"/>
-      <c r="G27" s="6" t="n"/>
-      <c r="H27" s="6" t="n"/>
-      <c r="I27" s="6" t="n"/>
-      <c r="J27" s="6" t="n"/>
-      <c r="K27" s="6" t="n"/>
-      <c r="L27" s="6" t="n"/>
-      <c r="M27" s="6">
-        <f>SUM(M3:M26)</f>
-        <v/>
-      </c>
-      <c r="N27" s="6">
-        <f>SUM(N3:N26)</f>
-        <v/>
-      </c>
-      <c r="O27" s="6">
-        <f>SUM(O3:O26)</f>
-        <v/>
-      </c>
-      <c r="P27" s="6">
-        <f>SUM(P3:P26)</f>
-        <v/>
-      </c>
-      <c r="Q27" s="6">
-        <f>SUM(Q3:Q26)</f>
-        <v/>
-      </c>
-      <c r="R27" s="6">
-        <f>SUM(R3:R26)</f>
-        <v/>
-      </c>
-      <c r="S27" s="6">
-        <f>SUM(S3:S26)</f>
-        <v/>
-      </c>
-      <c r="T27" s="6">
-        <f>SUM(T3:T26)</f>
-        <v/>
-      </c>
-      <c r="U27" s="6">
-        <f>SUM(U3:U26)</f>
-        <v/>
+      <c r="H29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x3 </t>
+        </is>
+      </c>
+      <c r="I29" s="4" t="inlineStr">
+        <is>
+          <t>20260917</t>
+        </is>
+      </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>SMS CORPORATION CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MODIFIED TAPIOCA STARCH </t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>NEED VERY CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M29" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="N29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T29" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U29" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="30" ht="13" customHeight="1">
-      <c r="A30" s="7" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C30" s="7" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260901071</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>NSSJ</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>2607S</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>202609220800</t>
+        </is>
+      </c>
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>THLKR</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>IDJKT</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx3 20'x1 </t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>20260917</t>
+        </is>
+      </c>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>TE CONNECTIVITY MANUFACTURING (THAILAND) CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>AUTOMOTIVE PART</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="P30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U30" s="4" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="31" ht="13" customHeight="1">
       <c r="A31" s="4" t="inlineStr">
         <is>
+          <t>HASLS22260901155</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>HAB</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>2611N</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>202609270600</t>
+        </is>
+      </c>
+      <c r="E31" s="4" t="inlineStr">
+        <is>
+          <t>THSRP</t>
+        </is>
+      </c>
+      <c r="F31" s="4" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>CNSHA</t>
+        </is>
+      </c>
+      <c r="H31" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx4 </t>
+        </is>
+      </c>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>20260916</t>
+        </is>
+      </c>
+      <c r="J31" s="4" t="inlineStr">
+        <is>
+          <t>VAST OCEAN CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>PP RECYCLE PELLET</t>
+        </is>
+      </c>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>RQST CONTAINER 32.5 TONS</t>
+        </is>
+      </c>
+      <c r="M31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T31" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U31" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" ht="13" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260901272</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>SWMM</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>202609221300</t>
+        </is>
+      </c>
+      <c r="E32" s="4" t="inlineStr"/>
+      <c r="F32" s="4" t="inlineStr">
+        <is>
+          <t>THBKK</t>
+        </is>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
+          <t>JPIYM</t>
+        </is>
+      </c>
+      <c r="H32" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x2 </t>
+        </is>
+      </c>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>20260917</t>
+        </is>
+      </c>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>SCG INTERNATIONAL CORPORATION CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>COPPER SCRAP</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>RQST Container clean and strong , Load by Folk lift</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U32" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" ht="13" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260901444</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>SWMM</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>202609221300</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr"/>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>THBKK</t>
+        </is>
+      </c>
+      <c r="G33" s="4" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H33" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx1 </t>
+        </is>
+      </c>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>20260917</t>
+        </is>
+      </c>
+      <c r="J33" s="4" t="inlineStr">
+        <is>
+          <t>SIAM KRAFT INDUSTRY CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K33" s="4" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O33" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T33" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U33" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" ht="13" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>HASLS22260901445</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>SWMM</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>202609221300</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr"/>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>THBKK</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>20260917</t>
+        </is>
+      </c>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>SIAM KRAFT INDUSTRY CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>PAPER</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M34" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U34" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" ht="13" customHeight="1">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B35" s="6" t="n"/>
+      <c r="C35" s="6" t="n"/>
+      <c r="D35" s="6" t="n"/>
+      <c r="E35" s="6" t="n"/>
+      <c r="F35" s="6" t="n"/>
+      <c r="G35" s="6" t="n"/>
+      <c r="H35" s="6" t="n"/>
+      <c r="I35" s="6" t="n"/>
+      <c r="J35" s="6" t="n"/>
+      <c r="K35" s="6" t="n"/>
+      <c r="L35" s="6" t="n"/>
+      <c r="M35" s="6">
+        <f>SUM(M3:M34)</f>
+        <v/>
+      </c>
+      <c r="N35" s="6">
+        <f>SUM(N3:N34)</f>
+        <v/>
+      </c>
+      <c r="O35" s="6">
+        <f>SUM(O3:O34)</f>
+        <v/>
+      </c>
+      <c r="P35" s="6">
+        <f>SUM(P3:P34)</f>
+        <v/>
+      </c>
+      <c r="Q35" s="6">
+        <f>SUM(Q3:Q34)</f>
+        <v/>
+      </c>
+      <c r="R35" s="6">
+        <f>SUM(R3:R34)</f>
+        <v/>
+      </c>
+      <c r="S35" s="6">
+        <f>SUM(S3:S34)</f>
+        <v/>
+      </c>
+      <c r="T35" s="6">
+        <f>SUM(T3:T34)</f>
+        <v/>
+      </c>
+      <c r="U35" s="6">
+        <f>SUM(U3:U34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" ht="13" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B38" s="7" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C38" s="7" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="13" customHeight="1">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
           <t>B.C. DEPOT CO.,LTD. ( Bang-Na KM.18)</t>
         </is>
       </c>
-      <c r="B31" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="C31" s="4" t="n">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="32" ht="13" customHeight="1">
-      <c r="A32" s="6" t="inlineStr">
+      <c r="B39" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="C39" s="4" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="40" ht="13" customHeight="1">
+      <c r="A40" s="6" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B32" s="6" t="n">
-        <v>24</v>
-      </c>
-      <c r="C32" s="6" t="n">
-        <v>85</v>
+      <c r="B40" s="6" t="n">
+        <v>32</v>
+      </c>
+      <c r="C40" s="6" t="n">
+        <v>100</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A2:U26"/>
+  <autoFilter ref="A2:U34"/>
   <mergeCells count="1">
     <mergeCell ref="A1:U1"/>
   </mergeCells>

</xml_diff>

<commit_message>
Fix column autofit: remove the 10-char floor that kept columns wide
The autofit width had a floor of 10 + padding of 2, which forced
short columns (VSL, GP22, POR, ...) to stay much wider than their
actual content — defeating the "tight to character count" request.
Floor is now 1 and padding 1, so width genuinely tracks the
longest value/header per column. ORG CUST/COMMODITY/TRAFFIC ORDER
still keep their fixed wide widths.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - B.C. DEPOT CO.,LTD. ( Bang-Na KM.18).xlsx
+++ b/output/bkg pending - B.C. DEPOT CO.,LTD. ( Bang-Na KM.18).xlsx
@@ -495,27 +495,27 @@
   <dimension ref="A1:U40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="5" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
     <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="10" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="10" customWidth="1" min="18" max="18"/>
-    <col width="10" customWidth="1" min="19" max="19"/>
-    <col width="10" customWidth="1" min="20" max="20"/>
-    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="5" customWidth="1" min="13" max="13"/>
+    <col width="5" customWidth="1" min="14" max="14"/>
+    <col width="5" customWidth="1" min="15" max="15"/>
+    <col width="5" customWidth="1" min="16" max="16"/>
+    <col width="5" customWidth="1" min="17" max="17"/>
+    <col width="5" customWidth="1" min="18" max="18"/>
+    <col width="5" customWidth="1" min="19" max="19"/>
+    <col width="5" customWidth="1" min="20" max="20"/>
+    <col width="5" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="13" customHeight="1">

</xml_diff>

<commit_message>
Update reports with 10-15-PD data
Regenerated from the full daily export "10-15-PD.xls" (2,583 rows):
126 BK No outstanding, 314 containers across 6 depots (UNITHAI and
YJC files removed as they have no data in this list). No rows
flagged for missing Pickup Name.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - B.C. DEPOT CO.,LTD. ( Bang-Na KM.18).xlsx
+++ b/output/bkg pending - B.C. DEPOT CO.,LTD. ( Bang-Na KM.18).xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -43,7 +43,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -53,11 +53,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002E75B6"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFF00"/>
       </patternFill>
     </fill>
     <fill>
@@ -97,7 +92,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -105,13 +100,10 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -479,17 +471,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U31"/>
+  <dimension ref="A1:U27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="4" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
     <col width="6" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
@@ -615,33 +607,37 @@
     <row r="2" ht="13" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260701285</t>
+          <t>HASLS22260900516</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>SWIC</t>
+          <t>YSVY</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2608S</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>202610150600</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr"/>
+          <t>202610220430</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>THLKR</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -651,22 +647,22 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>20261009</t>
+          <t>20261014</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>SINGHA WORLDWIDE INTERNATIONAL CO., LTD.</t>
+          <t>HYMOLD (THAILAND) LIMITED</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>LEMON SODA</t>
+          <t>FERRO SILICON MAGNESIUM</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>please put the container on the bottom of the vessel. Please pay careful attention to lift on/lift off at CY</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
@@ -700,68 +696,68 @@
     <row r="3" ht="13" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260801364</t>
+          <t>HASLS22260901128</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>SWIC</t>
+          <t>YSVY</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2608S</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>202610150600</t>
+          <t>202610220430</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>20261009</t>
+          <t>20261015</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>CROWN FOOD PACKAGING (THAILAND) PUBLIC COMPANY LIMITED</t>
+          <t>THAI PLASPAC PUBLIC CO.,LTD.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>EMPTY CAN</t>
+          <t>PLATIC CAP</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>REQUEST CLEAN CONTAINER</t>
+          <t>REQUEST GOOD &amp; CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="N3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O3" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="P3" s="2" t="n">
         <v>0</v>
@@ -785,12 +781,12 @@
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260900218</t>
+          <t>HASLS22260902010</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SWIC</t>
+          <t>SWAT</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -800,7 +796,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>202610150600</t>
+          <t>202611020100</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
@@ -811,42 +807,42 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>KRPUS</t>
+          <t>HKHKG</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx6 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>20261003</t>
+          <t>20260926</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>THAI ASAHI CO., LTD.</t>
+          <t>COSMOS BREWERY (THAILAND) CO.,LTD.</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">POTATO STARCH </t>
+          <t xml:space="preserve">BOTTLED CHANG BEER </t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>Grade A and food grade container</t>
+          <t>REQ. GOOD, CLEAN &amp; DRY GRADE A CONTAINER. PLEASE DO NOT CHANGE VESSEL AND PAPERLESS CODE</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O4" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P4" s="2" t="n">
         <v>0</v>
@@ -870,53 +866,57 @@
     <row r="5" ht="13" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901365</t>
+          <t>HASLS22260902173</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>SWIC</t>
+          <t>HMVY</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>202610150600</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr"/>
+          <t>202610252330</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>THSRP</t>
+        </is>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>CNSHA</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx5 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>20261009</t>
+          <t>20261015</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>EXCEL ENTECH CO.,LTD.</t>
+          <t>IDEC ASIA (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>PARTS OF MACHINERY</t>
+          <t>CONTACT BLOCK / ELECTRONIC PART</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
@@ -931,7 +931,7 @@
         <v>0</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="P5" s="2" t="n">
         <v>0</v>
@@ -955,22 +955,22 @@
     <row r="6" ht="13" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901617</t>
+          <t>HASLS22260902347</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>KJT</t>
+          <t>SWAL</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>202610181900</t>
+          <t>202610210900</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -981,7 +981,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -991,22 +991,22 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>20261009</t>
+          <t>20261015</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>THAI OTSUKA PHARMACEUTICAL CO., LTD.</t>
+          <t>EVEREST TEXTILE (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>MEDICAL</t>
+          <t>FABRIC</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>GOOD &amp; CLEAN CONT. , NO SMELL</t>
+          <t>Request clean container</t>
         </is>
       </c>
       <c r="M6" s="2" t="n">
@@ -1040,22 +1040,22 @@
     <row r="7" ht="13" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901619</t>
+          <t>HASLS22260902356</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>KJT</t>
+          <t>CMA</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2615N</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>202610181900</t>
+          <t>202610231400</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr"/>
@@ -1066,42 +1066,42 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>CNSHK</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>20261009</t>
+          <t>20261015</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>THAI OTSUKA PHARMACEUTICAL CO., LTD.</t>
+          <t>THAIMAN INDUSTRIES CO., LTD.</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>MEDICAL</t>
+          <t>POLYAMIDE 66 TEXTURED YARN</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>GOOD &amp; CLEAN CONT. , NO SMELL</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O7" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="N7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="P7" s="2" t="n">
         <v>0</v>
@@ -1125,70 +1125,72 @@
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901669</t>
+          <t>HASLS22260902449</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>SWIC</t>
+          <t>HMVY</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>202610150600</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr"/>
+          <t>202610252330</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>THSRP</t>
+        </is>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>CNSHA</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x7 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>20261009</t>
+          <t>20261015</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>THANAKORN VEGETABLE OIL PRODUCTS CO., LTD.</t>
+          <t>MITANI TRADING (THAILAND) CO.,LTD.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>SOYBEAN OIL</t>
+          <t>TWO WAY CAP</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>**APPROVAL BY MR.M.J CHANG DD.30/09/2026* *FLEXIBAG ONDECK*
-**APPRSurvey : 20226-10-09 , Pickup : 2026-10-10
- REQUEST STRONG, CLEAN, FOOD GRADE CNTR</t>
+          <t>GOOD AND CLEAN</t>
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="N8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P8" s="2" t="n">
         <v>0</v>
@@ -1212,22 +1214,22 @@
     <row r="9" ht="13" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901687</t>
+          <t>HASLS22260902581</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>SWIC</t>
+          <t>HAHM</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>202610150600</t>
+          <t>202610262300</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr"/>
@@ -1238,17 +1240,17 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>JPFKY</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx10 </t>
+          <t xml:space="preserve">20'x4 </t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>20261008</t>
+          <t>20261014</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1258,22 +1260,22 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>CABON BLACK</t>
+          <t>CARBON BLACK (NON DG)</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>*Clean container / No rust / No hole / No sharp surface inside areas in container.</t>
+          <t>CLEAN CONTAINER GRADE A</t>
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O9" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P9" s="2" t="n">
         <v>0</v>
@@ -1297,22 +1299,22 @@
     <row r="10" ht="13" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901726</t>
+          <t>HASLS22260902583</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>SWIC</t>
+          <t>HAHM</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>202610150600</t>
+          <t>202610262300</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr"/>
@@ -1323,42 +1325,42 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>KRKAN</t>
+          <t>JPFKY</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx2 </t>
+          <t xml:space="preserve">20'x8 </t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>20261009</t>
+          <t>20261015</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>THAI ASAHI CO., LTD.</t>
+          <t>BIRLA CARBON (THAILAND) PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">POTATO STARCH </t>
+          <t>CARBON BLACK (NON DG)</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Grade A and food grade container</t>
+          <t>CLEAN CONTAINER GRADE A</t>
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="N10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O10" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P10" s="2" t="n">
         <v>0</v>
@@ -1380,109 +1382,109 @@
       </c>
     </row>
     <row r="11" ht="13" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
-        <is>
-          <t>HASLS22260901813</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>KMTP</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>2612N</t>
-        </is>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
-        <is>
-          <t>202610141200</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22260902611</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>SWAL</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>202610210900</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G11" s="3" t="inlineStr">
-        <is>
-          <t>HKHKG</t>
-        </is>
-      </c>
-      <c r="H11" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R40Hx1 </t>
-        </is>
-      </c>
-      <c r="I11" s="3" t="inlineStr">
-        <is>
-          <t>20261008</t>
-        </is>
-      </c>
-      <c r="J11" s="3" t="inlineStr">
-        <is>
-          <t>KIBUN (THAILAND) CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K11" s="3" t="inlineStr">
-        <is>
-          <t>FROZEN IMITATION CRAB MEAT//1604.20</t>
-        </is>
-      </c>
-      <c r="L11" s="3" t="inlineStr">
-        <is>
-          <t>RF45REx1 (Temp -20.0℃ / Vent Close)</t>
-        </is>
-      </c>
-      <c r="M11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="3" t="n">
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>KRINC</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>20261015</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>UNICORD PUBLIC COMPANY LIMITED</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>PET FOOD</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="R11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U11" s="3" t="n">
+      <c r="N11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T11" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U11" s="2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12" ht="13" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901972</t>
+          <t>HASLS22260902753</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>KJT</t>
+          <t>CMA</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2615N</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>202610181900</t>
+          <t>202610231400</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
@@ -1493,7 +1495,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>TWKEL</t>
+          <t>HKHKG</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
@@ -1503,22 +1505,22 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>20261007</t>
+          <t>20261014</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>SMS CORPORATION CO., LTD.</t>
+          <t>SUREE INTERFOODS CO., LTD.</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">MODIFIED TAPIOCA STARCH </t>
+          <t>FOODSTUFFS</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>NEED VERY CLEAN CONTAINER</t>
+          <t>Good dry and clean container</t>
         </is>
       </c>
       <c r="M12" s="2" t="n">
@@ -1552,22 +1554,22 @@
     <row r="13" ht="13" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902010</t>
+          <t>HASLS22261000001</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>SWAT</t>
+          <t>HAHM</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>202611010400</t>
+          <t>202610262300</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
@@ -1578,42 +1580,42 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>JPMYJ</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>20260926</t>
+          <t>20261015</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>COSMOS BREWERY (THAILAND) CO.,LTD.</t>
+          <t>MULFRO (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">BOTTLED CHANG BEER </t>
+          <t>DRIED SALTED JELLY FISH</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>REQ. GOOD, CLEAN &amp; DRY GRADE A CONTAINER. PLEASE DO NOT CHANGE VESSEL AND PAPERLESS CODE</t>
+          <t>CLEAN, UNDER DECK, RQST CNTR GRADE A MAX 32.5 TONS</t>
         </is>
       </c>
       <c r="M13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="N13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="P13" s="2" t="n">
         <v>0</v>
@@ -1637,22 +1639,22 @@
     <row r="14" ht="13" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902181</t>
+          <t>HASLS22261000145</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>SWBT</t>
+          <t>KMGY</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>2616N</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>202610151900</t>
+          <t>202610231600</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr"/>
@@ -1663,42 +1665,42 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>KRINC</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx8 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>20261006</t>
+          <t>20261015</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>BIRLA CARBON (THAILAND) PUBLIC COMPANY LIMITED</t>
+          <t>MAHANAVA CO.,LTD.</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>CABON BLACK</t>
+          <t>FOODSTUFF</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>/ No rust / No hole / No sharp surface inside areas in container</t>
+          <t>REQ. GOOD AND CLEAN CONTAINER, NO SMELL, NO RUST, NO HOLE, FOOD GRADE</t>
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N14" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O14" s="2" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="P14" s="2" t="n">
         <v>0</v>
@@ -1722,22 +1724,22 @@
     <row r="15" ht="13" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902194</t>
+          <t>HASLS22261000159</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>PGPO</t>
+          <t>SWMM</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>202610151200</t>
+          <t>202610230900</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
@@ -1753,37 +1755,37 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx30 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>20261007</t>
+          <t>20261014</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>METRO PARTICLE CO., LTD.</t>
+          <t>K.P.FOODS CO., LTD.</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>PARTICLE BOARD</t>
+          <t>BISCUIT</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>RQST CNTR UPGRADE 32.50 TONS</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P15" s="2" t="n">
         <v>0</v>
@@ -1807,68 +1809,72 @@
     <row r="16" ht="13" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902207</t>
+          <t>HASLS22261000220</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>SWMM</t>
+          <t>HMVY</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>202610211900</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr"/>
+          <t>202610252330</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>THSRP</t>
+        </is>
+      </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>JPKSM</t>
+          <t>CNSHA</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x6 </t>
+          <t xml:space="preserve">40Hx1 20'x1 </t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>20261009</t>
+          <t>20261014</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>GENERAL MILLS CORPORATION LIMITED</t>
+          <t>INNOVALUES PRECISION (THAILAND) LTD.</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">TAPIOCA HARD PELLETS </t>
+          <t>AUTOMOTIVE PARTS</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>Request well clean and dry cntrs ,</t>
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O16" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P16" s="2" t="n">
         <v>0</v>
@@ -1892,12 +1898,12 @@
     <row r="17" ht="13" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902247</t>
+          <t>HASLS22261000425</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>PGPO</t>
+          <t>SKOR</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1907,7 +1913,7 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>202610151200</t>
+          <t>202610230100</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
@@ -1918,42 +1924,42 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>HKHKG</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>20261009</t>
+          <t>20261015</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>GENERAL CANDY CO., LTD.</t>
+          <t>NIPPN FOODS CORPORATION (THAILAND) LTD.</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>CANDY</t>
+          <t>RAW MATERIALS FOR MISTER DONUT &amp; FOODS</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>REQUEST CONTAINER GOOD AND FOOD GRADE</t>
+          <t>**GOOD AND CLEAN CONTAINER FOR FOOD (MISTER DONUT &amp; FOODS)</t>
         </is>
       </c>
       <c r="M17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N17" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O17" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P17" s="2" t="n">
         <v>0</v>
@@ -1977,22 +1983,22 @@
     <row r="18" ht="13" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902525</t>
+          <t>HASLS22261000536</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>SWIC</t>
+          <t>SKOR</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>202610150600</t>
+          <t>202610230100</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr"/>
@@ -2003,32 +2009,33 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>JPOSA</t>
+          <t>HKHKG</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx1 20'x1 </t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>20261009</t>
+          <t>20261014</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>NEW SOLUTION CO.,LTD</t>
+          <t>NISSIN FOODS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>COPPER SCRAP</t>
+          <t>INSTANT NOODLES BAG TYPE THAI SIGNATURE SERIES</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>CLEAN AND DRY CONTAINER</t>
+          <t>FOOD GRADE CONTAINER / GOOD AND CLEAN CONTAINER / NO LEAK
+SHIPPER : NI</t>
         </is>
       </c>
       <c r="M18" s="2" t="n">
@@ -2038,7 +2045,7 @@
         <v>0</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P18" s="2" t="n">
         <v>0</v>
@@ -2062,68 +2069,72 @@
     <row r="19" ht="13" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902531</t>
+          <t>HASLS22261000625</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>KJT</t>
+          <t>YSVY</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2608S</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>202610181900</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr"/>
+          <t>202610220430</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>THLKR</t>
+        </is>
+      </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>TWKEL</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>20261009</t>
+          <t>20261015</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>DZQ CO.,LTD.</t>
+          <t>Y.R.C. TEXTILE CO., LTD.</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>FRUIT JUICE, FOODSTUFF</t>
+          <t>TEXTILE</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>Food Grade, Dry, Clean, Good Container, No Rust, No Hole</t>
+          <t>GOOD AND CLEAN ONTAINER</t>
         </is>
       </c>
       <c r="M19" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N19" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O19" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P19" s="2" t="n">
         <v>0</v>
@@ -2147,12 +2158,12 @@
     <row r="20" ht="13" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902658</t>
+          <t>HASLS22261000857</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>SWIC</t>
+          <t>KJT</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -2162,7 +2173,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>202610150600</t>
+          <t>202610191100</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
@@ -2173,42 +2184,42 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>TWKEL</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x4 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>20261008</t>
+          <t>20261015</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>LAM SOON (THAILAND) PUBLIC COMPANY LIMITED</t>
+          <t>CHANG YI TRADING CO.,L TD</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>WHEAT FLOUR</t>
+          <t>FOODSTUFFS</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>REQUEST CLEAN AND GOOD CONTAINER ONLY</t>
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P20" s="2" t="n">
         <v>0</v>
@@ -2230,529 +2241,189 @@
       </c>
     </row>
     <row r="21" ht="13" customHeight="1">
-      <c r="A21" s="3" t="inlineStr">
-        <is>
-          <t>HASLS22260902791</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>SWIC</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22261001171</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>KJT</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>2611N</t>
         </is>
       </c>
-      <c r="D21" s="3" t="inlineStr">
-        <is>
-          <t>202610150600</t>
-        </is>
-      </c>
-      <c r="E21" s="3" t="inlineStr"/>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>202610191100</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>THBKK</t>
         </is>
       </c>
-      <c r="G21" s="3" t="inlineStr">
-        <is>
-          <t>RUVVO</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R40Hx7 </t>
-        </is>
-      </c>
-      <c r="I21" s="3" t="inlineStr">
-        <is>
-          <t>20261009</t>
-        </is>
-      </c>
-      <c r="J21" s="3" t="inlineStr">
-        <is>
-          <t>VENTE TRADE CO.,LTD.</t>
-        </is>
-      </c>
-      <c r="K21" s="3" t="inlineStr">
-        <is>
-          <t>CANNED PINEAPPLES</t>
-        </is>
-      </c>
-      <c r="L21" s="3" t="inlineStr">
-        <is>
-          <t>(TEMP : +18'C / VENT CLOSE)</t>
-        </is>
-      </c>
-      <c r="M21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="O21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q21" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="R21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T21" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="U21" s="3" t="n">
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>TWKEL</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx1 </t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>20261015</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>DELTA ELECTRIC (THAILAND) CO.,LTD.</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>ELECTRONICS COMPONENT</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U21" s="2" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22" ht="13" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22261000064</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>SWBT</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="inlineStr">
-        <is>
-          <t>2616N</t>
-        </is>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>202610151900</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>20261009</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
-        <is>
-          <t>GENERAL STARCH LIMITED</t>
-        </is>
-      </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>MODIFIED TAPIOCA STARCH</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>CLEAN / FOOD GRADE CONTAINER, NO HOLE, NO SMELL , WITHOUT ANY OIL STAIN</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N22" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q22" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R22" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S22" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T22" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U22" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" ht="13" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22261000079</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>SWBT</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="inlineStr">
-        <is>
-          <t>2616N</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>202610151900</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G23" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I23" s="2" t="inlineStr">
-        <is>
-          <t>20261009</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>NARA GLOBALCO., LTD.</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>MODELING CLAY</t>
-        </is>
-      </c>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>RQS CLEAN &amp; GOOD CONTAINER CONDITION.</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T23" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U23" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" ht="13" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22261000099</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>SWBT</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>2616N</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>202610151900</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G24" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40Hx1 </t>
-        </is>
-      </c>
-      <c r="I24" s="2" t="inlineStr">
-        <is>
-          <t>20261009</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr">
-        <is>
-          <t>ASIAN-PACIFIC CAN CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>COMMODITY : EMPTY CAN AND LID HS CODE : 7310.21 AND 8309.90</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O24" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="P24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U24" s="2" t="n">
-        <v>0</v>
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n"/>
+      <c r="C22" s="3" t="n"/>
+      <c r="D22" s="3" t="n"/>
+      <c r="E22" s="3" t="n"/>
+      <c r="F22" s="3" t="n"/>
+      <c r="G22" s="3" t="n"/>
+      <c r="H22" s="3" t="n"/>
+      <c r="I22" s="3" t="n"/>
+      <c r="J22" s="3" t="n"/>
+      <c r="K22" s="3" t="n"/>
+      <c r="L22" s="3" t="n"/>
+      <c r="M22" s="3">
+        <f>SUM(M2:M21)</f>
+        <v/>
+      </c>
+      <c r="N22" s="3">
+        <f>SUM(N2:N21)</f>
+        <v/>
+      </c>
+      <c r="O22" s="3">
+        <f>SUM(O2:O21)</f>
+        <v/>
+      </c>
+      <c r="P22" s="3">
+        <f>SUM(P2:P21)</f>
+        <v/>
+      </c>
+      <c r="Q22" s="3">
+        <f>SUM(Q2:Q21)</f>
+        <v/>
+      </c>
+      <c r="R22" s="3">
+        <f>SUM(R2:R21)</f>
+        <v/>
+      </c>
+      <c r="S22" s="3">
+        <f>SUM(S2:S21)</f>
+        <v/>
+      </c>
+      <c r="T22" s="3">
+        <f>SUM(T2:T21)</f>
+        <v/>
+      </c>
+      <c r="U22" s="3">
+        <f>SUM(U2:U21)</f>
+        <v/>
       </c>
     </row>
     <row r="25" ht="13" customHeight="1">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22261000681</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>KMTP</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="inlineStr">
-        <is>
-          <t>2612N</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>202610141200</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G25" s="2" t="inlineStr">
-        <is>
-          <t>KRPUS</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">40Hx1 </t>
-        </is>
-      </c>
-      <c r="I25" s="2" t="inlineStr">
-        <is>
-          <t>20261009</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr">
-        <is>
-          <t>IRONMAN 4X4 (THAILAND) LTD.</t>
-        </is>
-      </c>
-      <c r="K25" s="2" t="inlineStr">
-        <is>
-          <t>AUTOMOTIVE PARTS</t>
-        </is>
-      </c>
-      <c r="L25" s="2" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O25" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="P25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U25" s="2" t="n">
-        <v>0</v>
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
       </c>
     </row>
     <row r="26" ht="13" customHeight="1">
-      <c r="A26" s="4" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B26" s="4" t="n"/>
-      <c r="C26" s="4" t="n"/>
-      <c r="D26" s="4" t="n"/>
-      <c r="E26" s="4" t="n"/>
-      <c r="F26" s="4" t="n"/>
-      <c r="G26" s="4" t="n"/>
-      <c r="H26" s="4" t="n"/>
-      <c r="I26" s="4" t="n"/>
-      <c r="J26" s="4" t="n"/>
-      <c r="K26" s="4" t="n"/>
-      <c r="L26" s="4" t="n"/>
-      <c r="M26" s="4">
-        <f>SUM(M2:M25)</f>
-        <v/>
-      </c>
-      <c r="N26" s="4">
-        <f>SUM(N2:N25)</f>
-        <v/>
-      </c>
-      <c r="O26" s="4">
-        <f>SUM(O2:O25)</f>
-        <v/>
-      </c>
-      <c r="P26" s="4">
-        <f>SUM(P2:P25)</f>
-        <v/>
-      </c>
-      <c r="Q26" s="4">
-        <f>SUM(Q2:Q25)</f>
-        <v/>
-      </c>
-      <c r="R26" s="4">
-        <f>SUM(R2:R25)</f>
-        <v/>
-      </c>
-      <c r="S26" s="4">
-        <f>SUM(S2:S25)</f>
-        <v/>
-      </c>
-      <c r="T26" s="4">
-        <f>SUM(T2:T25)</f>
-        <v/>
-      </c>
-      <c r="U26" s="4">
-        <f>SUM(U2:U25)</f>
-        <v/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>B.C. DEPOT CO.,LTD. ( Bang-Na KM.18)</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>32</v>
       </c>
     </row>
-    <row r="29" ht="13" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="13" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>B.C. DEPOT CO.,LTD. ( Bang-Na KM.18)</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="C30" s="2" t="n">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="31" ht="13" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
+    <row r="27" ht="13" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B31" s="4" t="n">
-        <v>24</v>
-      </c>
-      <c r="C31" s="4" t="n">
-        <v>72</v>
+      <c r="B27" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>32</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U25"/>
+  <autoFilter ref="A1:U21"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update reports with 10-20-PD data
Regenerated from the full daily export "10-20-PD - Copy.xls"
(2,961 rows): 114 BK No outstanding, 308 containers across the
standard 6 depots. No rows flagged for missing Pickup Name.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - B.C. DEPOT CO.,LTD. ( Bang-Na KM.18).xlsx
+++ b/output/bkg pending - B.C. DEPOT CO.,LTD. ( Bang-Na KM.18).xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$27</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:U33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -607,12 +607,12 @@
     <row r="2" ht="13" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260900516</t>
+          <t>HASLS22260900492</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>YSVY</t>
+          <t>NSSJ</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -622,7 +622,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>202610220430</t>
+          <t>202610290200</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -642,37 +642,37 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>20261014</t>
+          <t>20261017</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>HYMOLD (THAILAND) LIMITED</t>
+          <t>THAI PLASPAC PUBLIC CO.,LTD.</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>FERRO SILICON MAGNESIUM</t>
+          <t>PLASTIC CAP</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>**REQUEST CLEAN AND GOOD CONTAINER</t>
         </is>
       </c>
       <c r="M2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="N2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="P2" s="2" t="n">
         <v>0</v>
@@ -696,12 +696,12 @@
     <row r="3" ht="13" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901128</t>
+          <t>HASLS22260901189</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>YSVY</t>
+          <t>KMSU</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -711,10 +711,14 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>202610220430</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr"/>
+          <t>202611012100</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>THLKR</t>
+        </is>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>THLCH</t>
@@ -727,37 +731,37 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x4 </t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>20261015</t>
+          <t>20261020</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>THAI PLASPAC PUBLIC CO.,LTD.</t>
+          <t>NORITAKE SCG PLASTER CO., LTD.</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>PLATIC CAP</t>
+          <t>MOULDING PLASTER</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>REQUEST GOOD &amp; CLEAN CONTAINER</t>
+          <t>Request good and clean cont., no oil, no rusty</t>
         </is>
       </c>
       <c r="M3" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="N3" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P3" s="2" t="n">
         <v>0</v>
@@ -781,22 +785,22 @@
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902010</t>
+          <t>HASLS22260901383</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>SWAT</t>
+          <t>KMBK</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>202611020100</t>
+          <t>202610260700</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
@@ -807,36 +811,36 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">20'x10 </t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>20260926</t>
+          <t>20261020</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>COSMOS BREWERY (THAILAND) CO.,LTD.</t>
+          <t>SCG INTERNATIONAL CORPORATION CO., LTD.</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">BOTTLED CHANG BEER </t>
+          <t>WHITE CLINKER</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>REQ. GOOD, CLEAN &amp; DRY GRADE A CONTAINER. PLEASE DO NOT CHANGE VESSEL AND PAPERLESS CODE</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -866,62 +870,58 @@
     <row r="5" ht="13" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902173</t>
+          <t>HASLS22260901723</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>HMVY</t>
+          <t>HAHM</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>202610252330</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>THSRP</t>
-        </is>
-      </c>
+          <t>202610271500</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>THLCH</t>
+          <t>THBKK</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>KRKAN</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">40Hx4 </t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>20261015</t>
+          <t>20261020</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>IDEC ASIA (THAILAND) CO., LTD.</t>
+          <t>THAI ASAHI CO., LTD.</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>CONTACT BLOCK / ELECTRONIC PART</t>
+          <t xml:space="preserve">POTATO STARCH </t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>Grade A and food grade container</t>
         </is>
       </c>
       <c r="M5" s="2" t="n">
@@ -931,7 +931,7 @@
         <v>0</v>
       </c>
       <c r="O5" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="P5" s="2" t="n">
         <v>0</v>
@@ -955,22 +955,22 @@
     <row r="6" ht="13" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902347</t>
+          <t>HASLS22260902010</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>SWAL</t>
+          <t>SWDN</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>202610210900</t>
+          <t>202610312100</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -981,7 +981,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>HKHKG</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -991,22 +991,22 @@
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>20261015</t>
+          <t>20260926</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>EVEREST TEXTILE (THAILAND) CO., LTD.</t>
+          <t>COSMOS BREWERY (THAILAND) CO.,LTD.</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>FABRIC</t>
+          <t xml:space="preserve">BOTTLED CHANG BEER </t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Request clean container</t>
+          <t>REQ. GOOD, CLEAN &amp; DRY GRADE A CONTAINER. PLEASE DO NOT CHANGE VESSEL AND PAPERLESS CODE</t>
         </is>
       </c>
       <c r="M6" s="2" t="n">
@@ -1040,68 +1040,73 @@
     <row r="7" ht="13" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902356</t>
+          <t>HASLS22260902116</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>CMA</t>
+          <t>NSSJ</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2615N</t>
+          <t>2608S</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>202610231400</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr"/>
+          <t>202610290200</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>THLKR</t>
+        </is>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>CNSHK</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>20261015</t>
+          <t>20261020</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>THAIMAN INDUSTRIES CO., LTD.</t>
+          <t>THAI PLASPAC PUBLIC CO.,LTD.</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>POLYAMIDE 66 TEXTURED YARN</t>
+          <t>PLATIC CAP</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>**REQUEST CLEAN AND GOOD CONTAINER**
+**REQUEST FREE TIME 14 DAYS COMBINE AT DESTINATION**</t>
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P7" s="2" t="n">
         <v>0</v>
@@ -1125,27 +1130,27 @@
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902449</t>
+          <t>HASLS22260902534</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>HMVY</t>
+          <t>KMSU</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2608S</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>202610252330</t>
+          <t>202611012100</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>THSRP</t>
+          <t>THLKR</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -1155,42 +1160,42 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>20261015</t>
+          <t>20261020</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>MITANI TRADING (THAILAND) CO.,LTD.</t>
+          <t>NORITAKE SCG PLASTER CO., LTD.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>TWO WAY CAP</t>
+          <t>MOULDING PLASTER</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN</t>
+          <t>good and clean cont., no oil, no rusty</t>
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P8" s="2" t="n">
         <v>0</v>
@@ -1214,62 +1219,66 @@
     <row r="9" ht="13" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902581</t>
+          <t>HASLS22260902697</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>HAHM</t>
+          <t>KMSU</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2608S</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>202610262300</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr"/>
+          <t>202611012100</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>THLKR</t>
+        </is>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>JPFKY</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x4 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>20261014</t>
+          <t>20261020</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>BIRLA CARBON (THAILAND) PUBLIC COMPANY LIMITED</t>
+          <t>ORFFA (THAILAND) COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>CARBON BLACK (NON DG)</t>
+          <t>EXCENTIAL SELENIUM</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>CLEAN CONTAINER GRADE A</t>
+          <t>REQUEST CONTAINR GOOD AND CLEAN</t>
         </is>
       </c>
       <c r="M9" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N9" s="2" t="n">
         <v>0</v>
@@ -1299,62 +1308,66 @@
     <row r="10" ht="13" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902583</t>
+          <t>HASLS22260902798</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>HAHM</t>
+          <t>KMSU</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2608S</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>202610262300</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr"/>
+          <t>202611012100</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>THLKR</t>
+        </is>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>JPFKY</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x8 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>20261015</t>
+          <t>20261020</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>BIRLA CARBON (THAILAND) PUBLIC COMPANY LIMITED</t>
+          <t>ORFFA (THAILAND) COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>CARBON BLACK (NON DG)</t>
+          <t>EXCENTIAL SELENIUM</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>CLEAN CONTAINER GRADE A</t>
+          <t>REQUEST CONTAINR GOOD AND CLEAN</t>
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="N10" s="2" t="n">
         <v>0</v>
@@ -1384,22 +1397,22 @@
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902611</t>
+          <t>HASLS22260902837</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>SWAL</t>
+          <t>HAHM</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>202610210900</t>
+          <t>202610271500</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr"/>
@@ -1410,42 +1423,42 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>KRINC</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx2 </t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>20261015</t>
+          <t>20261016</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>UNICORD PUBLIC COMPANY LIMITED</t>
+          <t>MEGAKLEEN PRODUCT CO.,LTD</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>PET FOOD</t>
+          <t>JET LIQUID</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>Request CNTR 32.5 TONS / Request Good and No Leakage Container</t>
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P11" s="2" t="n">
         <v>0</v>
@@ -1469,22 +1482,22 @@
     <row r="12" ht="13" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902753</t>
+          <t>HASLS22261000459</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>CMA</t>
+          <t>HAHM</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2615N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>202610231400</t>
+          <t>202610271500</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
@@ -1495,42 +1508,42 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx10 </t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>20261014</t>
+          <t>20261019</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>SUREE INTERFOODS CO., LTD.</t>
+          <t>BIRLA CARBON (THAILAND) PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>FOODSTUFFS</t>
+          <t>CABON BLACK</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Good dry and clean container</t>
+          <t>**Clean container / No rust / No hole / No sharp surface inside areas in container.</t>
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="P12" s="2" t="n">
         <v>0</v>
@@ -1554,12 +1567,12 @@
     <row r="13" ht="13" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261000001</t>
+          <t>HASLS22261000623</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>HAHM</t>
+          <t>SWIC</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1569,7 +1582,7 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>202610262300</t>
+          <t>202611100000</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr"/>
@@ -1580,7 +1593,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>JPMYJ</t>
+          <t>JPTHS</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1590,22 +1603,22 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>20261015</t>
+          <t>20261016</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>MULFRO (THAILAND) CO., LTD.</t>
+          <t>BIRLA CARBON (THAILAND) PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>DRIED SALTED JELLY FISH</t>
+          <t>CARBON BLACK (NON DG)</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>CLEAN, UNDER DECK, RQST CNTR GRADE A MAX 32.5 TONS</t>
+          <t>CLEAN CONTAINER GRADE A</t>
         </is>
       </c>
       <c r="M13" s="2" t="n">
@@ -1639,65 +1652,69 @@
     <row r="14" ht="13" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261000145</t>
+          <t>HASLS22261000672</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>KMGY</t>
+          <t>HAB</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>202610231600</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr"/>
+          <t>202610282300</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>THSRP</t>
+        </is>
+      </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>KRINC</t>
+          <t>CNSHA</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40'x1 </t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>20261015</t>
+          <t>20261019</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>MAHANAVA CO.,LTD.</t>
+          <t>BJC GLASS PREMIUM COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>FOODSTUFF</t>
+          <t>GLASS BOTTLE</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>REQ. GOOD AND CLEAN CONTAINER, NO SMELL, NO RUST, NO HOLE, FOOD GRADE</t>
+          <t>NEED GOOD CONTAINER</t>
         </is>
       </c>
       <c r="M14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="N14" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="O14" s="2" t="n">
         <v>0</v>
@@ -1724,22 +1741,22 @@
     <row r="15" ht="13" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261000159</t>
+          <t>HASLS22261000726</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>SWMM</t>
+          <t>KMBK</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>202610230900</t>
+          <t>202610260700</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
@@ -1755,22 +1772,22 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>20261014</t>
+          <t>20261019</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>K.P.FOODS CO., LTD.</t>
+          <t>TRILLION INDUSTRIES LIMITED</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>BISCUIT</t>
+          <t>PART MACHINE</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1779,13 +1796,13 @@
         </is>
       </c>
       <c r="M15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O15" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="N15" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O15" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="P15" s="2" t="n">
         <v>0</v>
@@ -1809,66 +1826,62 @@
     <row r="16" ht="13" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261000220</t>
+          <t>HASLS22261000931</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>HMVY</t>
+          <t>KMBK</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>202610252330</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>THSRP</t>
-        </is>
-      </c>
+          <t>202610260700</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>THLCH</t>
+          <t>THBKK</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 20'x1 </t>
+          <t xml:space="preserve">40Hx2 </t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>20261014</t>
+          <t>20261020</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>INNOVALUES PRECISION (THAILAND) LTD.</t>
+          <t>OTANI RADIAL CO., LTD.</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>AUTOMOTIVE PARTS</t>
+          <t>TIRES</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Request well clean and dry cntrs ,</t>
+          <t>REQUEST CONTAINER GOOD GRADE</t>
         </is>
       </c>
       <c r="M16" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N16" s="2" t="n">
         <v>0</v>
@@ -1898,22 +1911,22 @@
     <row r="17" ht="13" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261000425</t>
+          <t>HASLS22261001005</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>SKOR</t>
+          <t>KMGY</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>202610230100</t>
+          <t>202610240200</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
@@ -1934,22 +1947,22 @@
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>20261015</t>
+          <t>20261020</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>NIPPN FOODS CORPORATION (THAILAND) LTD.</t>
+          <t>J &amp; B SIAM MARKETING CO.,LTD.</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>RAW MATERIALS FOR MISTER DONUT &amp; FOODS</t>
+          <t>FOODSTUFFS</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>**GOOD AND CLEAN CONTAINER FOR FOOD (MISTER DONUT &amp; FOODS)</t>
+          <t>GOOD &amp; CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M17" s="2" t="n">
@@ -1983,59 +1996,62 @@
     <row r="18" ht="13" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261000536</t>
+          <t>HASLS22261001026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>SKOR</t>
+          <t>NSSJ</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2608S</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>202610230100</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr"/>
+          <t>202610290200</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>THLKR</t>
+        </is>
+      </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 20'x1 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>20261014</t>
+          <t>20261020</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>NISSIN FOODS (THAILAND) CO., LTD.</t>
+          <t>THAI TORAY SYNTHETICS  CO., LTD.</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>INSTANT NOODLES BAG TYPE THAI SIGNATURE SERIES</t>
+          <t>PLASTIC RESIN HS CODE 391110</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>FOOD GRADE CONTAINER / GOOD AND CLEAN CONTAINER / NO LEAK
-SHIPPER : NI</t>
+          <t>REQ.CONTAINER MUST BE IN GOOD CONDITION,NO HOLES,NO EXCESSIVE SPLINTERS ON THE FLOOR,NO HUMIDITY,THE FLOOR IS NOT SAGGING,THE FLOOR IS NOT SAGGING</t>
         </is>
       </c>
       <c r="M18" s="2" t="n">
@@ -2045,7 +2061,7 @@
         <v>0</v>
       </c>
       <c r="O18" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P18" s="2" t="n">
         <v>0</v>
@@ -2069,27 +2085,27 @@
     <row r="19" ht="13" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261000625</t>
+          <t>HASLS22261001079</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>YSVY</t>
+          <t>HMVY</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>2608S</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>202610220430</t>
+          <t>202610271300</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>THLKR</t>
+          <t>THSRP</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -2099,42 +2115,42 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>IDJKT</t>
+          <t>CNSHA</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>20261015</t>
+          <t>20261020</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>Y.R.C. TEXTILE CO., LTD.</t>
+          <t>DOCKWEILER ASIA CO., LTD.</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>TEXTILE</t>
+          <t>STAINLESS STEEL TUBE</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN ONTAINER</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="N19" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O19" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="P19" s="2" t="n">
         <v>0</v>
@@ -2158,68 +2174,68 @@
     <row r="20" ht="13" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261000857</t>
+          <t>HASLS22261001105</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>KJT</t>
+          <t>SWMM</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2610N</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>202610191100</t>
+          <t>202610251730</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>TWKEL</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>20261015</t>
+          <t>20261019</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>CHANG YI TRADING CO.,L TD</t>
+          <t>JONG STIT CO., LTD.</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>FOODSTUFFS</t>
+          <t>FABRIC</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>REQUEST CLEAN AND GOOD CONTAINER ONLY</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P20" s="2" t="n">
         <v>0</v>
@@ -2243,22 +2259,22 @@
     <row r="21" ht="13" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261001171</t>
+          <t>HASLS22261001272</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>KJT</t>
+          <t>HAHM</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>2611N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>202610191100</t>
+          <t>202610271500</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
@@ -2269,7 +2285,7 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>TWKEL</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -2279,17 +2295,17 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>20261015</t>
+          <t>20261020</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>DELTA ELECTRIC (THAILAND) CO.,LTD.</t>
+          <t>APEX CIRCUIT (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>ELECTRONICS COMPONENT</t>
+          <t>PRINTED CIRCUIT BOARD</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
@@ -2326,104 +2342,630 @@
       </c>
     </row>
     <row r="22" ht="13" customHeight="1">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="3" t="n"/>
-      <c r="J22" s="3" t="n"/>
-      <c r="K22" s="3" t="n"/>
-      <c r="L22" s="3" t="n"/>
-      <c r="M22" s="3">
-        <f>SUM(M2:M21)</f>
-        <v/>
-      </c>
-      <c r="N22" s="3">
-        <f>SUM(N2:N21)</f>
-        <v/>
-      </c>
-      <c r="O22" s="3">
-        <f>SUM(O2:O21)</f>
-        <v/>
-      </c>
-      <c r="P22" s="3">
-        <f>SUM(P2:P21)</f>
-        <v/>
-      </c>
-      <c r="Q22" s="3">
-        <f>SUM(Q2:Q21)</f>
-        <v/>
-      </c>
-      <c r="R22" s="3">
-        <f>SUM(R2:R21)</f>
-        <v/>
-      </c>
-      <c r="S22" s="3">
-        <f>SUM(S2:S21)</f>
-        <v/>
-      </c>
-      <c r="T22" s="3">
-        <f>SUM(T2:T21)</f>
-        <v/>
-      </c>
-      <c r="U22" s="3">
-        <f>SUM(U2:U21)</f>
-        <v/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22261001306</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>HMVY</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>202610271300</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>THSRP</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>CNSHA</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx1 20'x1 </t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>20261020</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>AVERY DENNISON (THAILAND) LTD.</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>SELF ADHESIVE MATERIAL</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Special Remark : Request well clean and dry cntrs ,</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U22" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" ht="13" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22261001309</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>HMVY</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>202610271300</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>THSRP</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>CNSHA</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>20261020</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>YUSEN LOGISTICS (THAILAND) CO.,LTD.</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>PRINTER FOR INDUSTRY</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T23" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U23" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" ht="13" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22261001354</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>HMVY</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>202610271300</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>THSRP</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>CNSHA</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx2 </t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>20261020</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>THAIGO LOGISTICS CO.,LTD</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>PC/ABS RECYCLE PELLET</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>RQST CNTR 32.5 TONS // 40'HQ</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="P24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U24" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="25" ht="13" customHeight="1">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22261001378</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>HMVY</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>2609N</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>202610271300</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>THSRP</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>THLCH</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>CNSHA</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">40Hx1 </t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>20261020</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>VAST OCEAN CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>POM RECYCLE PELLET</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>RQST CNTR 32.5 TONS // 40'HQ</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U25" s="2" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="26" ht="13" customHeight="1">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>HASLS22261001582</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>KMBK</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>2613N</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>202611160000</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>THBKK</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>20261012</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>BANPONG TAPIOCA FLOUR INDUSTRIAL CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FOOD FLOUR </t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U26" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" ht="13" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>HASLS22261001584</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>DJCF</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>0154N</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>202611230900</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>THBKK</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>VNSGN</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">20'x1 </t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>20261020</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>BANPONG TAPIOCA FLOUR INDUSTRIAL CO., LTD.</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FOOD FLOUR </t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>GOOD AND CLEAN CONTAINER</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="U27" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" ht="13" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n"/>
+      <c r="C28" s="3" t="n"/>
+      <c r="D28" s="3" t="n"/>
+      <c r="E28" s="3" t="n"/>
+      <c r="F28" s="3" t="n"/>
+      <c r="G28" s="3" t="n"/>
+      <c r="H28" s="3" t="n"/>
+      <c r="I28" s="3" t="n"/>
+      <c r="J28" s="3" t="n"/>
+      <c r="K28" s="3" t="n"/>
+      <c r="L28" s="3" t="n"/>
+      <c r="M28" s="3">
+        <f>SUM(M2:M27)</f>
+        <v/>
+      </c>
+      <c r="N28" s="3">
+        <f>SUM(N2:N27)</f>
+        <v/>
+      </c>
+      <c r="O28" s="3">
+        <f>SUM(O2:O27)</f>
+        <v/>
+      </c>
+      <c r="P28" s="3">
+        <f>SUM(P2:P27)</f>
+        <v/>
+      </c>
+      <c r="Q28" s="3">
+        <f>SUM(Q2:Q27)</f>
+        <v/>
+      </c>
+      <c r="R28" s="3">
+        <f>SUM(R2:R27)</f>
+        <v/>
+      </c>
+      <c r="S28" s="3">
+        <f>SUM(S2:S27)</f>
+        <v/>
+      </c>
+      <c r="T28" s="3">
+        <f>SUM(T2:T27)</f>
+        <v/>
+      </c>
+      <c r="U28" s="3">
+        <f>SUM(U2:U27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="13" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="13" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
           <t>B.C. DEPOT CO.,LTD. ( Bang-Na KM.18)</t>
         </is>
       </c>
-      <c r="B26" s="2" t="n">
-        <v>20</v>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="27" ht="13" customHeight="1">
-      <c r="A27" s="3" t="inlineStr">
+      <c r="B32" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="C32" s="2" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="33" ht="13" customHeight="1">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B27" s="3" t="n">
-        <v>20</v>
-      </c>
-      <c r="C27" s="3" t="n">
-        <v>32</v>
+      <c r="B33" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>46</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U21"/>
+  <autoFilter ref="A1:U27"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update reports with 10-21-PD data
Regenerated from the full daily export "10-21-PD.xls" (3,067
rows): 102 BK No outstanding, 265 containers across the standard
6 depots. No rows flagged for missing Pickup Name.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/bkg pending - B.C. DEPOT CO.,LTD. ( Bang-Na KM.18).xlsx
+++ b/output/bkg pending - B.C. DEPOT CO.,LTD. ( Bang-Na KM.18).xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pending" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$27</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Pending'!$A$1:$U$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U33"/>
+  <dimension ref="A1:U31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -481,7 +481,7 @@
     <col width="6" customWidth="1" min="5" max="5"/>
     <col width="6" customWidth="1" min="6" max="6"/>
     <col width="6" customWidth="1" min="7" max="7"/>
-    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="24" customWidth="1" min="11" max="11"/>
@@ -755,7 +755,7 @@
         </is>
       </c>
       <c r="M3" s="2" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N3" s="2" t="n">
         <v>0</v>
@@ -785,12 +785,12 @@
     <row r="4" ht="13" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260901383</t>
+          <t>HASLS22260901680</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>KMBK</t>
+          <t>HAHM</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -800,7 +800,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>202610260700</t>
+          <t>202610271500</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr"/>
@@ -811,36 +811,36 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>JPMIZ</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x10 </t>
+          <t xml:space="preserve">20'x5 </t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>20261020</t>
+          <t>20261021</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>SCG INTERNATIONAL CORPORATION CO., LTD.</t>
+          <t>FISHMEAL MARKETING DEVELOPMENT CO., LTD.</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>WHITE CLINKER</t>
+          <t>THAILAND STEAM DRIED FISHMEAL</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>**APPROVED BY MJ CHANG DD.23/09/26** DG22GPx5 (CLS 9 / UN 2216)  GOOD CONDITION OF CONTAINER, LOADING GOODS INTO CONTAINERD BY FOLKLIFT</t>
         </is>
       </c>
       <c r="M4" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N4" s="2" t="n">
         <v>0</v>
@@ -955,12 +955,12 @@
     <row r="6" ht="13" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902010</t>
+          <t>HASLS22260901732</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>SWDN</t>
+          <t>SWAT</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -970,7 +970,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>202610312100</t>
+          <t>202611032300</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr"/>
@@ -981,42 +981,42 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>HKHKG</t>
+          <t>RUVVO</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>20260926</t>
+          <t>20261021</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>COSMOS BREWERY (THAILAND) CO.,LTD.</t>
+          <t>I.P. ONE COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">BOTTLED CHANG BEER </t>
+          <t>HYGIENE SOFTENER CONCENTRATE</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>REQ. GOOD, CLEAN &amp; DRY GRADE A CONTAINER. PLEASE DO NOT CHANGE VESSEL AND PAPERLESS CODE</t>
+          <t>RQST CNTR GRADE A</t>
         </is>
       </c>
       <c r="M6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="N6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="P6" s="2" t="n">
         <v>0</v>
@@ -1040,67 +1040,63 @@
     <row r="7" ht="13" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902116</t>
+          <t>HASLS22260901926</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>NSSJ</t>
+          <t>HAHM</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>2608S</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>202610290200</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>THLKR</t>
-        </is>
-      </c>
+          <t>202610271500</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>THLCH</t>
+          <t>THBKK</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>IDJKT</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">20'x20 </t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>20261020</t>
+          <t>20261021</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>THAI PLASPAC PUBLIC CO.,LTD.</t>
+          <t>THANAKORN VEGETABLE OIL PRODUCTS CO., LTD.</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>PLATIC CAP</t>
+          <t>SOYBEAN OIL</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>**REQUEST CLEAN AND GOOD CONTAINER**
-**REQUEST FREE TIME 14 DAYS COMBINE AT DESTINATION**</t>
+          <t>**APPROVED BY MJ CHANG DD.01/10/26***FLEXIBAG ONDECK*
+Survey : 2026-10-21, Pickup : 2026-10-22 REQUEST STRONG, CLEAN, FOOD GRADE CONTAINER</t>
         </is>
       </c>
       <c r="M7" s="2" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="N7" s="2" t="n">
         <v>0</v>
@@ -1130,37 +1126,33 @@
     <row r="8" ht="13" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902534</t>
+          <t>HASLS22260901996</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>KMSU</t>
+          <t>KMGY</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>2608S</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>202611012100</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>THLKR</t>
-        </is>
-      </c>
+          <t>202610240200</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>THLCH</t>
+          <t>THBKK</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>IDJKT</t>
+          <t>KRINC</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1170,26 +1162,27 @@
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>20261020</t>
+          <t>20261021</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>NORITAKE SCG PLASTER CO., LTD.</t>
+          <t>PANTAINORASINGH MANUFACTURER CO.,LTD.</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>MOULDING PLASTER</t>
+          <t>FOODSTUFFS</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>good and clean cont., no oil, no rusty</t>
+          <t>be in new condition, clean, have a flat surface with no beams, a smooth ceiling, and no leaks.
+It must also be rust-free, odorless, never used to sto</t>
         </is>
       </c>
       <c r="M8" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N8" s="2" t="n">
         <v>0</v>
@@ -1219,72 +1212,68 @@
     <row r="9" ht="13" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902697</t>
+          <t>HASLS22260902080</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>KMSU</t>
+          <t>HAHM</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>2608S</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>202611012100</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>THLKR</t>
-        </is>
-      </c>
+          <t>202610271500</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>THLCH</t>
+          <t>THBKK</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>IDJKT</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>20261020</t>
+          <t>20261021</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>ORFFA (THAILAND) COMPANY LIMITED</t>
+          <t>NIPRO (THAILAND) CORPORATION LIMITED</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>EXCENTIAL SELENIUM</t>
+          <t>MEDICAL PRODUCT</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>REQUEST CONTAINR GOOD AND CLEAN</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="N9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="P9" s="2" t="n">
         <v>0</v>
@@ -1308,7 +1297,7 @@
     <row r="10" ht="13" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902798</t>
+          <t>HASLS22260902534</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -1343,7 +1332,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">20'x2 </t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1353,21 +1342,21 @@
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>ORFFA (THAILAND) COMPANY LIMITED</t>
+          <t>NORITAKE SCG PLASTER CO., LTD.</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>EXCENTIAL SELENIUM</t>
+          <t>MOULDING PLASTER</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>REQUEST CONTAINR GOOD AND CLEAN</t>
+          <t>good and clean cont., no oil, no rusty</t>
         </is>
       </c>
       <c r="M10" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N10" s="2" t="n">
         <v>0</v>
@@ -1397,7 +1386,7 @@
     <row r="11" ht="13" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>HASLS22260902837</t>
+          <t>HASLS22260902583</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
@@ -1423,42 +1412,42 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>JPFKY</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx2 </t>
+          <t xml:space="preserve">20'x8 </t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>20261016</t>
+          <t>20261021</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>MEGAKLEEN PRODUCT CO.,LTD</t>
+          <t>BIRLA CARBON (THAILAND) PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>JET LIQUID</t>
+          <t>CARBON BLACK (NON DG)</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Request CNTR 32.5 TONS / Request Good and No Leakage Container</t>
+          <t>CLEAN CONTAINER GRADE A</t>
         </is>
       </c>
       <c r="M11" s="2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N11" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P11" s="2" t="n">
         <v>0</v>
@@ -1482,68 +1471,72 @@
     <row r="12" ht="13" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261000459</t>
+          <t>HASLS22260902697</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>HAHM</t>
+          <t>KMSU</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2608S</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>202610271500</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr"/>
+          <t>202611012100</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>THLKR</t>
+        </is>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx10 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>20261019</t>
+          <t>20261020</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>BIRLA CARBON (THAILAND) PUBLIC COMPANY LIMITED</t>
+          <t>ORFFA (THAILAND) COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>CABON BLACK</t>
+          <t>EXCENTIAL SELENIUM</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>**Clean container / No rust / No hole / No sharp surface inside areas in container.</t>
+          <t>REQUEST CONTAINR GOOD AND CLEAN</t>
         </is>
       </c>
       <c r="M12" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N12" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="P12" s="2" t="n">
         <v>0</v>
@@ -1567,68 +1560,72 @@
     <row r="13" ht="13" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261000623</t>
+          <t>HASLS22260902798</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>SWIC</t>
+          <t>KMSU</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2608S</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>202611100000</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr"/>
+          <t>202611012100</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>THLKR</t>
+        </is>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>THBKK</t>
+          <t>THLCH</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>JPTHS</t>
+          <t>IDJKT</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>20261016</t>
+          <t>20261020</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>BIRLA CARBON (THAILAND) PUBLIC COMPANY LIMITED</t>
+          <t>ORFFA (THAILAND) COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>CARBON BLACK (NON DG)</t>
+          <t>EXCENTIAL SELENIUM</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>CLEAN CONTAINER GRADE A</t>
+          <t>REQUEST CONTAINR GOOD AND CLEAN</t>
         </is>
       </c>
       <c r="M13" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N13" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O13" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P13" s="2" t="n">
         <v>0</v>
@@ -1652,12 +1649,12 @@
     <row r="14" ht="13" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261000672</t>
+          <t>HASLS22261000012</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>HAB</t>
+          <t>HAHM</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1667,54 +1664,51 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>202610282300</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>THSRP</t>
-        </is>
-      </c>
+          <t>202610271500</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>THLCH</t>
+          <t>THBKK</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40'x1 </t>
+          <t xml:space="preserve">20'x5 </t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>20261019</t>
+          <t>20261021</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>BJC GLASS PREMIUM COMPANY LIMITED</t>
+          <t>ICONS GLOBAL LOGISTICS CO., LTD.</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>GLASS BOTTLE</t>
+          <t>SOYBEAN OIL</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>NEED GOOD CONTAINER</t>
+          <t>** APPROVED BY MJ CHANG DD.01/10/26** *FLEXIBAG ONDECK*
+Survey : 2026-10-21</t>
         </is>
       </c>
       <c r="M14" s="2" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O14" s="2" t="n">
         <v>0</v>
@@ -1741,12 +1735,12 @@
     <row r="15" ht="13" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261000726</t>
+          <t>HASLS22261000387</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>KMBK</t>
+          <t>HAHM</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1756,7 +1750,7 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>202610260700</t>
+          <t>202610271500</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr"/>
@@ -1772,37 +1766,37 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>20261019</t>
+          <t>20261021</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>TRILLION INDUSTRIES LIMITED</t>
+          <t>TORAY TEXTILES (THAILAND) PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>PART MACHINE</t>
+          <t>FABRIC</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>Request clean container</t>
         </is>
       </c>
       <c r="M15" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N15" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O15" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P15" s="2" t="n">
         <v>0</v>
@@ -1826,12 +1820,12 @@
     <row r="16" ht="13" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261000931</t>
+          <t>HASLS22261000623</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>KMBK</t>
+          <t>SWIC</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1841,7 +1835,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>202610260700</t>
+          <t>202611100000</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr"/>
@@ -1852,32 +1846,32 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>JPTHS</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx2 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>20261020</t>
+          <t>20261016</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>OTANI RADIAL CO., LTD.</t>
+          <t>BIRLA CARBON (THAILAND) PUBLIC COMPANY LIMITED</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>TIRES</t>
+          <t>CARBON BLACK (NON DG)</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>REQUEST CONTAINER GOOD GRADE</t>
+          <t>CLEAN CONTAINER GRADE A</t>
         </is>
       </c>
       <c r="M16" s="2" t="n">
@@ -1911,7 +1905,7 @@
     <row r="17" ht="13" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261001005</t>
+          <t>HASLS22261000662</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
@@ -1942,37 +1936,37 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx1 </t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>20261020</t>
+          <t>20261021</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>J &amp; B SIAM MARKETING CO.,LTD.</t>
+          <t>PROMPT PLUS  CO.,LTD.</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>FOODSTUFFS</t>
+          <t>PRINTER</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>GOOD &amp; CLEAN CONTAINER</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="N17" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O17" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="P17" s="2" t="n">
         <v>0</v>
@@ -1996,72 +1990,68 @@
     <row r="18" ht="13" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261001026</t>
+          <t>HASLS22261000674</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>NSSJ</t>
+          <t>HAHM</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>2608S</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>202610290200</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>THLKR</t>
-        </is>
-      </c>
+          <t>202610271500</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>THLCH</t>
+          <t>THBKK</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>IDJKT</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx3 </t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>20261020</t>
+          <t>20261021</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>THAI TORAY SYNTHETICS  CO., LTD.</t>
+          <t>OTANI RADIAL CO., LTD.</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>PLASTIC RESIN HS CODE 391110</t>
+          <t>NEW TIRE</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>REQ.CONTAINER MUST BE IN GOOD CONDITION,NO HOLES,NO EXCESSIVE SPLINTERS ON THE FLOOR,NO HUMIDITY,THE FLOOR IS NOT SAGGING,THE FLOOR IS NOT SAGGING</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O18" s="2" t="n">
         <v>1</v>
-      </c>
-      <c r="N18" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O18" s="2" t="n">
-        <v>0</v>
       </c>
       <c r="P18" s="2" t="n">
         <v>0</v>
@@ -2085,37 +2075,33 @@
     <row r="19" ht="13" customHeight="1">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261001079</t>
+          <t>HASLS22261001289</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>HMVY</t>
+          <t>KMBK</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>202610271300</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>THSRP</t>
-        </is>
-      </c>
+          <t>202610260700</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>THLCH</t>
+          <t>THBKK</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>KRPUS</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -2125,17 +2111,17 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>20261020</t>
+          <t>20261021</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>DOCKWEILER ASIA CO., LTD.</t>
+          <t>NISSIN FOODS (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>STAINLESS STEEL TUBE</t>
+          <t>NISSIN INSTANT CUP NOODLES</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
@@ -2174,25 +2160,29 @@
     <row r="20" ht="13" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261001105</t>
+          <t>HASLS22261001354</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>SWMM</t>
+          <t>HMVY</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>2610N</t>
+          <t>2609N</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>202610251730</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
+          <t>202610271900</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>THSRP</t>
+        </is>
+      </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
           <t>THLCH</t>
@@ -2200,42 +2190,42 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>CNSHA</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">20'x1 </t>
+          <t xml:space="preserve">40Hx2 </t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>20261019</t>
+          <t>20261020</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>JONG STIT CO., LTD.</t>
+          <t>THAIGO LOGISTICS CO.,LTD</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>FABRIC</t>
+          <t>PC/ABS RECYCLE PELLET</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>RQST CNTR 32.5 TONS // 40'HQ</t>
         </is>
       </c>
       <c r="M20" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N20" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O20" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P20" s="2" t="n">
         <v>0</v>
@@ -2259,22 +2249,22 @@
     <row r="21" ht="13" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261001272</t>
+          <t>HASLS22261001564</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>HAHM</t>
+          <t>KMGY</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>2612N</t>
+          <t>2611N</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>202610271500</t>
+          <t>202610240200</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr"/>
@@ -2285,42 +2275,42 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>VNSGN</t>
+          <t>KRINC</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>20261020</t>
+          <t>20261021</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>APEX CIRCUIT (THAILAND) CO., LTD.</t>
+          <t>ANDAMAN JELLYFISH CO.,LTD.</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>PRINTED CIRCUIT BOARD</t>
+          <t>SALTED JELLYFISH</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
+          <t>UNDER DECK</t>
         </is>
       </c>
       <c r="M21" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N21" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O21" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P21" s="2" t="n">
         <v>0</v>
@@ -2344,62 +2334,58 @@
     <row r="22" ht="13" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261001306</t>
+          <t>HASLS22261001568</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>HMVY</t>
+          <t>SWVG</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2613N</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>202610271300</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>THSRP</t>
-        </is>
-      </c>
+          <t>202610282000</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>THLCH</t>
+          <t>THBKK</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>HKHKG</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 20'x1 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>20261020</t>
+          <t>20261021</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>AVERY DENNISON (THAILAND) LTD.</t>
+          <t>SIAM TIN FOOD PRODUCTS CO.,LTD.</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>SELF ADHESIVE MATERIAL</t>
+          <t>CANNED PET FOODS</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>Special Remark : Request well clean and dry cntrs ,</t>
+          <t>REQ : GOOD &amp; CLEAN / NOT SMELL CONTAINER (FOOD GRADE)</t>
         </is>
       </c>
       <c r="M22" s="2" t="n">
@@ -2409,7 +2395,7 @@
         <v>0</v>
       </c>
       <c r="O22" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P22" s="2" t="n">
         <v>0</v>
@@ -2433,37 +2419,33 @@
     <row r="23" ht="13" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261001309</t>
+          <t>HASLS22261001582</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>HMVY</t>
+          <t>KMBK</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2613N</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>202610271300</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>THSRP</t>
-        </is>
-      </c>
+          <t>202611160000</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>THLCH</t>
+          <t>THBKK</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2473,17 +2455,17 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>20261020</t>
+          <t>20261012</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>YUSEN LOGISTICS (THAILAND) CO.,LTD.</t>
+          <t>BANPONG TAPIOCA FLOUR INDUSTRIAL CO., LTD.</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>PRINTER FOR INDUSTRY</t>
+          <t xml:space="preserve">FOOD FLOUR </t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -2522,42 +2504,38 @@
     <row r="24" ht="13" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261001354</t>
+          <t>HASLS22261001584</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>HMVY</t>
+          <t>DJCF</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>0154N</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>202610271300</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>THSRP</t>
-        </is>
-      </c>
+          <t>202611232200</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>THLCH</t>
+          <t>THBKK</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx2 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -2567,27 +2545,27 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>THAIGO LOGISTICS CO.,LTD</t>
+          <t>BANPONG TAPIOCA FLOUR INDUSTRIAL CO., LTD.</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>PC/ABS RECYCLE PELLET</t>
+          <t xml:space="preserve">FOOD FLOUR </t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>RQST CNTR 32.5 TONS // 40'HQ</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M24" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N24" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O24" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="P24" s="2" t="n">
         <v>0</v>
@@ -2611,72 +2589,68 @@
     <row r="25" ht="13" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>HASLS22261001378</t>
+          <t>HASLS22261001619</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>HMVY</t>
+          <t>KMBK</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>2609N</t>
+          <t>2612N</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>202610271300</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>THSRP</t>
-        </is>
-      </c>
+          <t>202610260700</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr"/>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>THLCH</t>
+          <t>THBKK</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>CNSHA</t>
+          <t>VNSGN</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">40Hx1 </t>
+          <t xml:space="preserve">20'x1 </t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>20261020</t>
+          <t>20261021</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>VAST OCEAN CO., LTD.</t>
+          <t>FORMICA (THAILAND) CO., LTD.</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>POM RECYCLE PELLET</t>
+          <t>MELAMINE DECORATIVE SHEET</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>RQST CNTR 32.5 TONS // 40'HQ</t>
+          <t>GOOD AND CLEAN CONTAINER</t>
         </is>
       </c>
       <c r="M25" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N25" s="2" t="n">
         <v>0</v>
       </c>
       <c r="O25" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P25" s="2" t="n">
         <v>0</v>
@@ -2698,274 +2672,104 @@
       </c>
     </row>
     <row r="26" ht="13" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22261001582</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>KMBK</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>2613N</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>202611160000</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>20261012</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr">
-        <is>
-          <t>BANPONG TAPIOCA FLOUR INDUSTRIAL CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FOOD FLOUR </t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U26" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" ht="13" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>HASLS22261001584</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>DJCF</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="inlineStr">
-        <is>
-          <t>0154N</t>
-        </is>
-      </c>
-      <c r="D27" s="2" t="inlineStr">
-        <is>
-          <t>202611230900</t>
-        </is>
-      </c>
-      <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>THBKK</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>VNSGN</t>
-        </is>
-      </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">20'x1 </t>
-        </is>
-      </c>
-      <c r="I27" s="2" t="inlineStr">
-        <is>
-          <t>20261020</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr">
-        <is>
-          <t>BANPONG TAPIOCA FLOUR INDUSTRIAL CO., LTD.</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FOOD FLOUR </t>
-        </is>
-      </c>
-      <c r="L27" s="2" t="inlineStr">
-        <is>
-          <t>GOOD AND CLEAN CONTAINER</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="P27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="U27" s="2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" ht="13" customHeight="1">
-      <c r="A28" s="3" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B28" s="3" t="n"/>
-      <c r="C28" s="3" t="n"/>
-      <c r="D28" s="3" t="n"/>
-      <c r="E28" s="3" t="n"/>
-      <c r="F28" s="3" t="n"/>
-      <c r="G28" s="3" t="n"/>
-      <c r="H28" s="3" t="n"/>
-      <c r="I28" s="3" t="n"/>
-      <c r="J28" s="3" t="n"/>
-      <c r="K28" s="3" t="n"/>
-      <c r="L28" s="3" t="n"/>
-      <c r="M28" s="3">
-        <f>SUM(M2:M27)</f>
+      <c r="B26" s="3" t="n"/>
+      <c r="C26" s="3" t="n"/>
+      <c r="D26" s="3" t="n"/>
+      <c r="E26" s="3" t="n"/>
+      <c r="F26" s="3" t="n"/>
+      <c r="G26" s="3" t="n"/>
+      <c r="H26" s="3" t="n"/>
+      <c r="I26" s="3" t="n"/>
+      <c r="J26" s="3" t="n"/>
+      <c r="K26" s="3" t="n"/>
+      <c r="L26" s="3" t="n"/>
+      <c r="M26" s="3">
+        <f>SUM(M2:M25)</f>
         <v/>
       </c>
-      <c r="N28" s="3">
-        <f>SUM(N2:N27)</f>
+      <c r="N26" s="3">
+        <f>SUM(N2:N25)</f>
         <v/>
       </c>
-      <c r="O28" s="3">
-        <f>SUM(O2:O27)</f>
+      <c r="O26" s="3">
+        <f>SUM(O2:O25)</f>
         <v/>
       </c>
-      <c r="P28" s="3">
-        <f>SUM(P2:P27)</f>
+      <c r="P26" s="3">
+        <f>SUM(P2:P25)</f>
         <v/>
       </c>
-      <c r="Q28" s="3">
-        <f>SUM(Q2:Q27)</f>
+      <c r="Q26" s="3">
+        <f>SUM(Q2:Q25)</f>
         <v/>
       </c>
-      <c r="R28" s="3">
-        <f>SUM(R2:R27)</f>
+      <c r="R26" s="3">
+        <f>SUM(R2:R25)</f>
         <v/>
       </c>
-      <c r="S28" s="3">
-        <f>SUM(S2:S27)</f>
+      <c r="S26" s="3">
+        <f>SUM(S2:S25)</f>
         <v/>
       </c>
-      <c r="T28" s="3">
-        <f>SUM(T2:T27)</f>
+      <c r="T26" s="3">
+        <f>SUM(T2:T25)</f>
         <v/>
       </c>
-      <c r="U28" s="3">
-        <f>SUM(U2:U27)</f>
+      <c r="U26" s="3">
+        <f>SUM(U2:U25)</f>
         <v/>
       </c>
     </row>
+    <row r="29" ht="13" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>Pickup Name</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>Number of Records</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Total Balance</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="13" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>B.C. DEPOT CO.,LTD. ( Bang-Na KM.18)</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>61</v>
+      </c>
+    </row>
     <row r="31" ht="13" customHeight="1">
-      <c r="A31" s="4" t="inlineStr">
-        <is>
-          <t>Pickup Name</t>
-        </is>
-      </c>
-      <c r="B31" s="4" t="inlineStr">
-        <is>
-          <t>Number of Records</t>
-        </is>
-      </c>
-      <c r="C31" s="4" t="inlineStr">
-        <is>
-          <t>Total Balance</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="13" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>B.C. DEPOT CO.,LTD. ( Bang-Na KM.18)</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="C32" s="2" t="n">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="33" ht="13" customHeight="1">
-      <c r="A33" s="3" t="inlineStr">
+      <c r="A31" s="3" t="inlineStr">
         <is>
           <t>สรุปยอดบุ๊คทั้งหมด</t>
         </is>
       </c>
-      <c r="B33" s="3" t="n">
-        <v>26</v>
-      </c>
-      <c r="C33" s="3" t="n">
-        <v>46</v>
+      <c r="B31" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="C31" s="3" t="n">
+        <v>61</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:U27"/>
+  <autoFilter ref="A1:U25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>